<commit_message>
feat(tcs): expand Type tagging — SM/CP complete, Admin/Buyer partial
Coverage delta:
  SM     107 → 243 (4/4 files, 97-100% each)  — COMPLETE
  CP     221 → 278 (6/6 files, 93-100% each)  — COMPLETE
  Admin  0   → 174 (Login 100%, Customers 74%; 9 files pending)
  Buyer  84  → 192 (Dashboard/KYC/Login/UnitDetails ~95%; 7 files pending)

Total explicit Type rows: ~887 / 1,728 (~51%).
Remaining files fall back to script's auto-inference heuristic.

Rate-limited agents will resume after 3pm IST reset to finish 16 files.

Regenerated all 4 Excel workbooks with richer type distributions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual-qa-repository/07-execution/TestCases-CPPortal.xlsx
+++ b/manual-qa-repository/07-execution/TestCases-CPPortal.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3069" uniqueCount="1470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3069" uniqueCount="1471">
   <si>
     <t>CHANNEL PARTNER PORTAL — MASTER TEST CASE DOCUMENT</t>
   </si>
@@ -97,7 +97,7 @@
     <t>Project Information</t>
   </si>
   <si>
-    <t>UI:16 · FUNC:29 · VAL:4 · BIZ:1 · INT:15 · API:1 · NEG:1</t>
+    <t>UI:18 · FUNC:6 · BIZ:10 · INT:17 · API:3 · EDGE:6 · NEG:7</t>
   </si>
   <si>
     <t>Project Information — 67 TCs</t>
@@ -3601,9 +3601,6 @@
     <t>CHANNEL PARTNER PORTAL — Project Information Test Cases</t>
   </si>
   <si>
-    <t>━━━━━━━━━━  UI TESTS  (16)  ━━━━━━━━━━</t>
-  </si>
-  <si>
     <t>CP_PROJ_001</t>
   </si>
   <si>
@@ -3709,18 +3706,6 @@
     <t>Video gallery renders with embedded players or thumbnails</t>
   </si>
   <si>
-    <t>CP_PROJ_009</t>
-  </si>
-  <si>
-    <t>Logged-out user redirected from project pages</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/about` directly in a fresh browser</t>
-  </si>
-  <si>
-    <t>Redirect to `/login`</t>
-  </si>
-  <si>
     <t>CP_PROJ_010</t>
   </si>
   <si>
@@ -3739,52 +3724,73 @@
     <t>Paragraphs describing project background, location, and developer are visible</t>
   </si>
   <si>
-    <t>CP_PROJ_011</t>
-  </si>
-  <si>
-    <t>About is read-only — no edit controls present</t>
-  </si>
-  <si>
-    <t>1. Inspect page for Edit / Save / Delete actions</t>
-  </si>
-  <si>
-    <t>No edit controls; content is read-only</t>
-  </si>
-  <si>
-    <t>CP_PROJ_016</t>
+    <t>CP_PROJ_012</t>
+  </si>
+  <si>
+    <t>Gallery</t>
+  </si>
+  <si>
+    <t>Gallery loads project photos in grid</t>
+  </si>
+  <si>
+    <t>Gallery page open</t>
+  </si>
+  <si>
+    <t>1. Scroll Gallery grid</t>
+  </si>
+  <si>
+    <t>Photos render in a grid layout; images load without 404s</t>
+  </si>
+  <si>
+    <t>CP_PROJ_013</t>
+  </si>
+  <si>
+    <t>Click a photo opens larger view</t>
+  </si>
+  <si>
+    <t>Gallery has at least one image</t>
+  </si>
+  <si>
+    <t>1. Click any thumbnail</t>
+  </si>
+  <si>
+    <t>Lightbox / modal opens displaying the full-size image with close control</t>
+  </si>
+  <si>
+    <t>CP_PROJ_015</t>
   </si>
   <si>
     <t>Amenities</t>
   </si>
   <si>
-    <t>Amenities content is read-only</t>
-  </si>
-  <si>
-    <t>Amenities open</t>
-  </si>
-  <si>
-    <t>1. Look for any input or edit action</t>
-  </si>
-  <si>
-    <t>No editable controls available</t>
-  </si>
-  <si>
-    <t>CP_PROJ_019</t>
+    <t>Amenities list renders with names</t>
+  </si>
+  <si>
+    <t>Amenities page open</t>
+  </si>
+  <si>
+    <t>1. Read items in the amenities list</t>
+  </si>
+  <si>
+    <t>Amenity names displayed; categories or icons present per Strapi configuration</t>
+  </si>
+  <si>
+    <t>CP_PROJ_017</t>
   </si>
   <si>
     <t>Documents</t>
   </si>
   <si>
-    <t>Documents are read-only — no upload control</t>
+    <t>RERA document is listed</t>
   </si>
   <si>
     <t>Documents page open</t>
   </si>
   <si>
-    <t>1. Look for any Upload / Delete control</t>
-  </si>
-  <si>
-    <t>No upload/edit controls visible — content fully read-only</t>
+    <t>1. Scan the document list</t>
+  </si>
+  <si>
+    <t>At least one entry labelled RERA Registration is present</t>
   </si>
   <si>
     <t>CP_PROJ_020</t>
@@ -3805,110 +3811,71 @@
     <t>Bullet/numbered list of key selling points renders as content</t>
   </si>
   <si>
-    <t>CP_PROJ_021</t>
-  </si>
-  <si>
-    <t>Key Points are read-only</t>
-  </si>
-  <si>
-    <t>1. Look for Edit/Add controls</t>
-  </si>
-  <si>
-    <t>No edit controls present</t>
-  </si>
-  <si>
-    <t>CP_PROJ_053</t>
-  </si>
-  <si>
-    <t>Key Points HTML content uses safe rendering (NOT dangerouslySetInnerHTML)</t>
-  </si>
-  <si>
-    <t>Strapi key-point contains `&lt;script&gt;alert(1)&lt;/script&gt;` string</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Key Points page
-2. Inspect DOM</t>
-  </si>
-  <si>
-    <t>Script tag rendered as escaped text (NOT executed). If it executes → file as XSS gap analogous to CP_PROJ_033 / CP-PI-004. Verify keyPoints uses safe text rendering.</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  FUNCTIONAL TESTS  (29)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_012</t>
-  </si>
-  <si>
-    <t>Gallery</t>
-  </si>
-  <si>
-    <t>Gallery loads project photos in grid</t>
-  </si>
-  <si>
-    <t>Gallery page open</t>
-  </si>
-  <si>
-    <t>1. Scroll Gallery grid</t>
-  </si>
-  <si>
-    <t>Photos render in a grid layout; images load without 404s</t>
-  </si>
-  <si>
-    <t>CP_PROJ_013</t>
-  </si>
-  <si>
-    <t>Click a photo opens larger view</t>
-  </si>
-  <si>
-    <t>Gallery has at least one image</t>
-  </si>
-  <si>
-    <t>1. Click any thumbnail</t>
-  </si>
-  <si>
-    <t>Lightbox / modal opens displaying the full-size image with close control</t>
-  </si>
-  <si>
-    <t>CP_PROJ_014</t>
-  </si>
-  <si>
-    <t>Empty Gallery shows placeholder</t>
-  </si>
-  <si>
-    <t>Strapi returns no images</t>
-  </si>
-  <si>
-    <t>1. Open Gallery</t>
-  </si>
-  <si>
-    <t>Empty-state message such as "No photos available yet" is displayed</t>
-  </si>
-  <si>
-    <t>CP_PROJ_015</t>
-  </si>
-  <si>
-    <t>Amenities list renders with names</t>
-  </si>
-  <si>
-    <t>Amenities page open</t>
-  </si>
-  <si>
-    <t>1. Read items in the amenities list</t>
-  </si>
-  <si>
-    <t>Amenity names displayed; categories or icons present per Strapi configuration</t>
-  </si>
-  <si>
-    <t>CP_PROJ_017</t>
-  </si>
-  <si>
-    <t>RERA document is listed</t>
-  </si>
-  <si>
-    <t>1. Scan the document list</t>
-  </si>
-  <si>
-    <t>At least one entry labelled RERA Registration is present</t>
+    <t>CP_PROJ_022</t>
+  </si>
+  <si>
+    <t>Videos</t>
+  </si>
+  <si>
+    <t>Videos page lists video thumbnails</t>
+  </si>
+  <si>
+    <t>Videos page open</t>
+  </si>
+  <si>
+    <t>1. Scroll list of videos</t>
+  </si>
+  <si>
+    <t>Video thumbnails or embeds render</t>
+  </si>
+  <si>
+    <t>CP_PROJ_035</t>
+  </si>
+  <si>
+    <t>Single-newline whitespace in `information` collapses (UX gap)</t>
+  </si>
+  <si>
+    <t>Author writes content with single newlines between sentences</t>
+  </si>
+  <si>
+    <t>1. Render Project Info page</t>
+  </si>
+  <si>
+    <t>Single `\n` is dropped; only `\n\n` converted to `&lt;br /&gt;&lt;br /&gt;` (CP-PI-009, projectInfo.jsx:14). Authors must use double-newline.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_038</t>
+  </si>
+  <si>
+    <t>About content renders double-newline as paragraph break</t>
+  </si>
+  <si>
+    <t>Strapi `information` field contains `Para A\n\nPara B`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Render About page
+2. Inspect rendered HTML</t>
+  </si>
+  <si>
+    <t>`\n\n` rendered as `&lt;br /&gt;&lt;br /&gt;`; single `\n` between sentences silently collapsed (CP-PI-009, projectInfo.jsx:14). Authors must use double-newlines for paragraph breaks.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_052</t>
+  </si>
+  <si>
+    <t>Long key-point text wraps without horizontal scroll</t>
+  </si>
+  <si>
+    <t>Strapi contains a key-point &gt;300 chars</t>
+  </si>
+  <si>
+    <t>1. Render Key Points page on desktop and mobile viewport</t>
+  </si>
+  <si>
+    <t>Text wraps within container; no horizontal scrollbar appears; layout intact across breakpoints.</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  FUNCTIONAL TESTS  (6)  ━━━━━━━━━━</t>
   </si>
   <si>
     <t>CP_PROJ_018</t>
@@ -3924,24 +3891,6 @@
   </si>
   <si>
     <t>Browser initiates download or opens the document in a new tab</t>
-  </si>
-  <si>
-    <t>CP_PROJ_022</t>
-  </si>
-  <si>
-    <t>Videos</t>
-  </si>
-  <si>
-    <t>Videos page lists video thumbnails</t>
-  </si>
-  <si>
-    <t>Videos page open</t>
-  </si>
-  <si>
-    <t>1. Scroll list of videos</t>
-  </si>
-  <si>
-    <t>Video thumbnails or embeds render</t>
   </si>
   <si>
     <t>CP_PROJ_023</t>
@@ -3979,6 +3928,75 @@
     <t>Same section page loads from the copied URL</t>
   </si>
   <si>
+    <t>CP_PROJ_042</t>
+  </si>
+  <si>
+    <t>About loads without redirect when CP session active</t>
+  </si>
+  <si>
+    <t>Valid CP JWT in client storage</t>
+  </si>
+  <si>
+    <t>1. Open `/project1/about` directly in a new tab</t>
+  </si>
+  <si>
+    <t>About page renders without redirect to `/login`; Strapi call fires once; no XR backend dependency for content (FSD §6.1).</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  BUSINESS RULE TESTS  (10)  ━━━━━━━━━━</t>
+  </si>
+  <si>
+    <t>CP_PROJ_011</t>
+  </si>
+  <si>
+    <t>About is read-only — no edit controls present</t>
+  </si>
+  <si>
+    <t>1. Inspect page for Edit / Save / Delete actions</t>
+  </si>
+  <si>
+    <t>No edit controls; content is read-only</t>
+  </si>
+  <si>
+    <t>CP_PROJ_016</t>
+  </si>
+  <si>
+    <t>Amenities content is read-only</t>
+  </si>
+  <si>
+    <t>Amenities open</t>
+  </si>
+  <si>
+    <t>1. Look for any input or edit action</t>
+  </si>
+  <si>
+    <t>No editable controls available</t>
+  </si>
+  <si>
+    <t>CP_PROJ_019</t>
+  </si>
+  <si>
+    <t>Documents are read-only — no upload control</t>
+  </si>
+  <si>
+    <t>1. Look for any Upload / Delete control</t>
+  </si>
+  <si>
+    <t>No upload/edit controls visible — content fully read-only</t>
+  </si>
+  <si>
+    <t>CP_PROJ_021</t>
+  </si>
+  <si>
+    <t>Key Points are read-only</t>
+  </si>
+  <si>
+    <t>1. Look for Edit/Add controls</t>
+  </si>
+  <si>
+    <t>No edit controls present</t>
+  </si>
+  <si>
     <t>CP_PROJ_026</t>
   </si>
   <si>
@@ -4008,6 +4026,338 @@
   </si>
   <si>
     <t>Both fetch identical content from `&lt;StrapiBase&gt;/api/projects/1?populate=deep`. There is NO CP-project assignment table — every CP sees the same project (CP-PI-003). Document.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_031</t>
+  </si>
+  <si>
+    <t>Project ID hardcoded to `1` regardless of env</t>
+  </si>
+  <si>
+    <t>UAT (backend projectId=2)</t>
+  </si>
+  <si>
+    <t>1. Inspect Strapi URL</t>
+  </si>
+  <si>
+    <t>URL = `&lt;StrapiBase&gt;/api/projects/1?populate=deep` (CP-PI-002, Urls.js:7). Mismatched with backend project resolution — drift if Strapi project 1 differs from backend project 2.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_036</t>
+  </si>
+  <si>
+    <t>No analytics / view tracking on project pages</t>
+  </si>
+  <si>
+    <t>CP browses project pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Browse all sections
+2. Check XR DB / logs for view tracking</t>
+  </si>
+  <si>
+    <t>No tracking exists in XR Portal (QA-Risk-10). If engagement metrics needed, file as gap.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_048</t>
+  </si>
+  <si>
+    <t>Amenities list is identical for Master CP and Member CP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as M, snapshot amenities list
+2. Login as N, snapshot amenities list
+3. Compare</t>
+  </si>
+  <si>
+    <t>Lists are byte-identical — Strapi has no per-CP scoping; no CP-project assignment table (CP-PI-003). Both fetch same `projects/1?populate=deep`.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_060</t>
+  </si>
+  <si>
+    <t>Videos page is identical for Master CP and Member CP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Login as M, list videos
+2. Login as N, list videos</t>
+  </si>
+  <si>
+    <t>Same video list both times — no per-CP scoping in Strapi (CP-PI-003). Confirms no project-assignment table on CP side.</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  INTEGRATION TESTS  (17)  ━━━━━━━━━━</t>
+  </si>
+  <si>
+    <t>CP_PROJ_025</t>
+  </si>
+  <si>
+    <t>Content reflects latest Strapi publish</t>
+  </si>
+  <si>
+    <t>Admin has published an update in Strapi CMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the affected section in CP portal
+2. Hard refresh</t>
+  </si>
+  <si>
+    <t>Updated content is visible reflecting the latest Strapi publish</t>
+  </si>
+  <si>
+    <t>CP_PROJ_030</t>
+  </si>
+  <si>
+    <t>Frontend fetches Strapi directly (no XR proxy)</t>
+  </si>
+  <si>
+    <t>CP logged in, network tab open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open `/project1/about`
+2. Inspect network requests</t>
+  </si>
+  <si>
+    <t>Direct `GET &lt;BaseURL&gt;/api/projects/1?populate=deep` to Strapi host. NO request to XR backend `/api/v1/*` for project content (Urls.js:7).</t>
+  </si>
+  <si>
+    <t>CP_PROJ_032</t>
+  </si>
+  <si>
+    <t>Strapi outage breaks CP project pages silently</t>
+  </si>
+  <si>
+    <t>Block Strapi URL in browser</t>
+  </si>
+  <si>
+    <t>1. Open `/project1/about`</t>
+  </si>
+  <si>
+    <t>Frontend fails to render — no XR-side circuit breaker / cache (CP-PI-007). UI may white-screen. Document accessibility implications.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_037</t>
+  </si>
+  <si>
+    <t>About section sources `information` field directly from Strapi</t>
+  </si>
+  <si>
+    <t>CP logged in; About page open; network tab visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to `/project1/about`
+2. Inspect network requests</t>
+  </si>
+  <si>
+    <t>A `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` is fired directly from the CP browser; About content renders from `data.attributes.information` field (CP-PI-002, Urls.js:7). No XR backend call for project content.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_041</t>
+  </si>
+  <si>
+    <t>About reflects latest Strapi publish without hard refresh delay</t>
+  </si>
+  <si>
+    <t>Admin updates `information` in Strapi and clicks Publish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CP performs hard refresh on `/project1/about` (Ctrl+Shift+R)
+2. Read content</t>
+  </si>
+  <si>
+    <t>Updated content appears immediately — no XR-side ISR/cache (CP-PI-007). Browser fetch hits Strapi live each load.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_043</t>
+  </si>
+  <si>
+    <t>Amenities list sourced from Strapi `amenities` relation</t>
+  </si>
+  <si>
+    <t>Amenities page open; network tab visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open `/project1/amenities`
+2. Inspect Strapi response</t>
+  </si>
+  <si>
+    <t>Amenity items rendered from `data.attributes.amenities.data[].attributes` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). Each item shows name + icon URL.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_044</t>
+  </si>
+  <si>
+    <t>Amenity icons load from Strapi asset URLs without 404s</t>
+  </si>
+  <si>
+    <t>Strapi amenities have published icon assets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Render Amenities list
+2. Observe icon image requests in network tab</t>
+  </si>
+  <si>
+    <t>Every icon URL (raw Strapi `attributes.url`) returns 200; no broken-image placeholders; unsigned URLs cacheable (CP-PI-005).</t>
+  </si>
+  <si>
+    <t>CP_PROJ_046</t>
+  </si>
+  <si>
+    <t>Strapi outage breaks Amenities section silently</t>
+  </si>
+  <si>
+    <t>Block Strapi host in browser DevTools</t>
+  </si>
+  <si>
+    <t>1. Open `/project1/amenities`</t>
+  </si>
+  <si>
+    <t>Frontend has NO XR-side fallback — section either white-screens or shows error boundary (CP-PI-007). No cached version served by XR backend. Document accessibility/UX gap.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_047</t>
+  </si>
+  <si>
+    <t>Amenities returns DRAFT entries via populate=deep (publish gating bug)</t>
+  </si>
+  <si>
+    <t>Admin creates an amenity in Strapi but does NOT publish it</t>
+  </si>
+  <si>
+    <t>1. Open Amenities page in CP</t>
+  </si>
+  <si>
+    <t>Verify whether draft amenity appears. `populate=deep` may include DRAFT + PUBLISHED unless `publicationState=live` is passed (CP-PI-008, QA-Risk-14). If DRAFT visible → document as bug.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_049</t>
+  </si>
+  <si>
+    <t>Key Points sourced from Strapi `keyPoints` field</t>
+  </si>
+  <si>
+    <t>Key Points page open; network tab visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open `/project1/keyPoints`
+2. Inspect Strapi response</t>
+  </si>
+  <si>
+    <t>List items rendered from `data.attributes.keyPoints` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). No XR backend route involved.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_050</t>
+  </si>
+  <si>
+    <t>Key Points renders ordered list with correct sequence from Strapi</t>
+  </si>
+  <si>
+    <t>Strapi has 5 key-point entries in defined order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Render Key Points page
+2. Read items top → bottom</t>
+  </si>
+  <si>
+    <t>Items render in the same order as the Strapi array; no client-side re-sort; numbering / bullets follow source ordering.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_054</t>
+  </si>
+  <si>
+    <t>Key Points reflects latest Strapi publish after hard refresh</t>
+  </si>
+  <si>
+    <t>Admin publishes a new key-point in Strapi</t>
+  </si>
+  <si>
+    <t>1. CP performs Ctrl+Shift+R on `/project1/keyPoints`</t>
+  </si>
+  <si>
+    <t>New point appears immediately — no XR-side cache (CP-PI-007). Browser request hits Strapi live.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_055</t>
+  </si>
+  <si>
+    <t>Videos list sourced from Strapi `videos` relation</t>
+  </si>
+  <si>
+    <t>Videos page open; network tab visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open `/project1/videos`
+2. Inspect Strapi response</t>
+  </si>
+  <si>
+    <t>Items rendered from `data.attributes.videos.data[]` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). Each item supplies a video URL/embed code + thumbnail.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_057</t>
+  </si>
+  <si>
+    <t>Video thumbnails load from Strapi asset URLs</t>
+  </si>
+  <si>
+    <t>At least 2 published videos in Strapi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Render Videos page
+2. Inspect each `&lt;img&gt;` request</t>
+  </si>
+  <si>
+    <t>Thumbnail URLs (raw Strapi asset) return 200; no 404s; unsigned URLs cacheable; same external-shareable trait as brochure assets (CP-PI-005).</t>
+  </si>
+  <si>
+    <t>CP_PROJ_058</t>
+  </si>
+  <si>
+    <t>Video embed plays without leaking CP session credentials</t>
+  </si>
+  <si>
+    <t>Video uses third-party embed (YouTube/Vimeo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click and play a video
+2. Inspect outbound requests in network tab</t>
+  </si>
+  <si>
+    <t>Requests go directly to third-party host; no XR JWT / cookies forwarded; embed renders inside iframe sandbox.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_063</t>
+  </si>
+  <si>
+    <t>Strapi DRAFT entries should not leak via `populate=deep`</t>
+  </si>
+  <si>
+    <t>Admin creates a DRAFT entry in any populated relation (gallery/videos/keyPoints/amenities) without publishing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open `/project1/&lt;section&gt;` as CP
+2. Compare visible items vs Strapi admin</t>
+  </si>
+  <si>
+    <t>Only PUBLISHED entries should render. If DRAFT appears → file as bug (CP-PI-008, QA-Risk-14). Fix is to add `publicationState=live` to Strapi URL.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_064</t>
+  </si>
+  <si>
+    <t>Hard refresh always fetches latest Strapi state (no XR cache)</t>
+  </si>
+  <si>
+    <t>Admin publishes a content edit in Strapi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CP triggers Ctrl+Shift+R on any project section
+2. Inspect network requests</t>
+  </si>
+  <si>
+    <t>A fresh `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` is fired (no 304 / cache-hit on XR side); response reflects newly published content (CP-PI-007). Confirms no XR-side ISR / caching.</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  API TESTS  (3)  ━━━━━━━━━━</t>
   </si>
   <si>
     <t>CP_PROJ_028</t>
@@ -4043,51 +4393,148 @@
     <t>403 — `cp` role NOT in `restrictTo('user', 'admin', 'sales_manager_admin', 'sales_manager')` (common.routes.js:8).</t>
   </si>
   <si>
-    <t>CP_PROJ_031</t>
-  </si>
-  <si>
-    <t>Project ID hardcoded to `1` regardless of env</t>
-  </si>
-  <si>
-    <t>UAT (backend projectId=2)</t>
-  </si>
-  <si>
-    <t>1. Inspect Strapi URL</t>
-  </si>
-  <si>
-    <t>URL = `&lt;StrapiBase&gt;/api/projects/1?populate=deep` (CP-PI-002, Urls.js:7). Mismatched with backend project resolution — drift if Strapi project 1 differs from backend project 2.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_036</t>
-  </si>
-  <si>
-    <t>No analytics / view tracking on project pages</t>
-  </si>
-  <si>
-    <t>CP browses project pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Browse all sections
-2. Check XR DB / logs for view tracking</t>
-  </si>
-  <si>
-    <t>No tracking exists in XR Portal (QA-Risk-10). If engagement metrics needed, file as gap.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_038</t>
-  </si>
-  <si>
-    <t>About content renders double-newline as paragraph break</t>
-  </si>
-  <si>
-    <t>Strapi `information` field contains `Para A\n\nPara B`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render About page
-2. Inspect rendered HTML</t>
-  </si>
-  <si>
-    <t>`\n\n` rendered as `&lt;br /&gt;&lt;br /&gt;`; single `\n` between sentences silently collapsed (CP-PI-009, projectInfo.jsx:14). Authors must use double-newlines for paragraph breaks.</t>
+    <t>CORRECTION — There is NO XR backend endpoint for CP project info</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  EDGE CASE TESTS  (6)  ━━━━━━━━━━</t>
+  </si>
+  <si>
+    <t>CP_PROJ_014</t>
+  </si>
+  <si>
+    <t>Empty Gallery shows placeholder</t>
+  </si>
+  <si>
+    <t>Strapi returns no images</t>
+  </si>
+  <si>
+    <t>1. Open Gallery</t>
+  </si>
+  <si>
+    <t>Empty-state message such as "No photos available yet" is displayed</t>
+  </si>
+  <si>
+    <t>CP_PROJ_040</t>
+  </si>
+  <si>
+    <t>About section shows empty placeholder when `information` is null</t>
+  </si>
+  <si>
+    <t>Strapi `information` field is null or empty string</t>
+  </si>
+  <si>
+    <t>1. Open About page</t>
+  </si>
+  <si>
+    <t>Page renders heading; body shows empty placeholder or no content paragraph (NOT a JS error or broken layout).</t>
+  </si>
+  <si>
+    <t>CP_PROJ_045</t>
+  </si>
+  <si>
+    <t>Empty Amenities list shows graceful placeholder</t>
+  </si>
+  <si>
+    <t>Strapi returns `amenities.data = []`</t>
+  </si>
+  <si>
+    <t>1. Open Amenities page</t>
+  </si>
+  <si>
+    <t>Friendly empty-state copy displayed (e.g., "No amenities published yet"); UI does not error; section heading still renders.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_051</t>
+  </si>
+  <si>
+    <t>Empty Key Points list shows placeholder</t>
+  </si>
+  <si>
+    <t>Strapi `keyPoints` array is empty</t>
+  </si>
+  <si>
+    <t>1. Open Key Points page</t>
+  </si>
+  <si>
+    <t>Page renders with heading and friendly empty-state copy (e.g., "No key points published yet"); no JS errors.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_056</t>
+  </si>
+  <si>
+    <t>Empty Videos list shows placeholder copy</t>
+  </si>
+  <si>
+    <t>Strapi returns no videos</t>
+  </si>
+  <si>
+    <t>1. Open Videos page</t>
+  </si>
+  <si>
+    <t>Empty-state copy (e.g., "No videos available yet"); section heading still renders; no broken layout.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_059</t>
+  </si>
+  <si>
+    <t>Broken/invalid video URL falls back gracefully</t>
+  </si>
+  <si>
+    <t>A Strapi video item has malformed URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Videos page
+2. Click the broken video</t>
+  </si>
+  <si>
+    <t>Embedded player shows its own error UI (or thumbnail with "Unavailable" overlay); page does not crash; other videos remain playable.</t>
+  </si>
+  <si>
+    <t>━━━━━━━━━━  NEGATIVE TESTS  (7)  ━━━━━━━━━━</t>
+  </si>
+  <si>
+    <t>CP_PROJ_009</t>
+  </si>
+  <si>
+    <t>Logged-out user redirected from project pages</t>
+  </si>
+  <si>
+    <t>1. Open `/project1/about` directly in a fresh browser</t>
+  </si>
+  <si>
+    <t>Redirect to `/login`</t>
+  </si>
+  <si>
+    <t>CP_PROJ_033</t>
+  </si>
+  <si>
+    <t>`information` field XSS via Strapi WYSIWYG (potential)</t>
+  </si>
+  <si>
+    <t>Admin can write to Strapi `information` field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Insert `&lt;script&gt;alert(1)&lt;/script&gt;` via Strapi admin
+2. Open `/project1/projectInfo`</t>
+  </si>
+  <si>
+    <t>Script executes in CP browser — frontend uses `dangerouslySetInnerHTML` without sanitization (CP-PI-004, projectInfo.jsx:14). Trust boundary depends entirely on Strapi authoring controls. Document as security gap.</t>
+  </si>
+  <si>
+    <t>CP_PROJ_034</t>
+  </si>
+  <si>
+    <t>Brochure URL is unsigned Strapi asset (shareable externally)</t>
+  </si>
+  <si>
+    <t>Project info page open with brochure published</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Copy brochure URL from `data.brochure.data.attributes.url`
+2. Open in incognito (no CP session)</t>
+  </si>
+  <si>
+    <t>PDF downloads without auth — raw Strapi URL, no presigned/expiry (CP-PI-005). Confirm with security if acceptable.</t>
   </si>
   <si>
     <t>CP_PROJ_039</t>
@@ -4106,122 +4553,20 @@
     <t>Script executes — frontend uses `dangerouslySetInnerHTML` without sanitization (CP-PI-004, projectInfo.jsx:14). KNOWN SECURITY GAP: trust boundary lies entirely with Strapi authoring controls.</t>
   </si>
   <si>
-    <t>CP_PROJ_042</t>
-  </si>
-  <si>
-    <t>About loads without redirect when CP session active</t>
-  </si>
-  <si>
-    <t>Valid CP JWT in client storage</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/about` directly in a new tab</t>
-  </si>
-  <si>
-    <t>About page renders without redirect to `/login`; Strapi call fires once; no XR backend dependency for content (FSD §6.1).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_045</t>
-  </si>
-  <si>
-    <t>Empty Amenities list shows graceful placeholder</t>
-  </si>
-  <si>
-    <t>Strapi returns `amenities.data = []`</t>
-  </si>
-  <si>
-    <t>1. Open Amenities page</t>
-  </si>
-  <si>
-    <t>Friendly empty-state copy displayed (e.g., "No amenities published yet"); UI does not error; section heading still renders.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_048</t>
-  </si>
-  <si>
-    <t>Amenities list is identical for Master CP and Member CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Login as M, snapshot amenities list
-2. Login as N, snapshot amenities list
-3. Compare</t>
-  </si>
-  <si>
-    <t>Lists are byte-identical — Strapi has no per-CP scoping; no CP-project assignment table (CP-PI-003). Both fetch same `projects/1?populate=deep`.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_051</t>
-  </si>
-  <si>
-    <t>Empty Key Points list shows placeholder</t>
-  </si>
-  <si>
-    <t>Strapi `keyPoints` array is empty</t>
-  </si>
-  <si>
-    <t>1. Open Key Points page</t>
-  </si>
-  <si>
-    <t>Page renders with heading and friendly empty-state copy (e.g., "No key points published yet"); no JS errors.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_052</t>
-  </si>
-  <si>
-    <t>Long key-point text wraps without horizontal scroll</t>
-  </si>
-  <si>
-    <t>Strapi contains a key-point &gt;300 chars</t>
-  </si>
-  <si>
-    <t>1. Render Key Points page on desktop and mobile viewport</t>
-  </si>
-  <si>
-    <t>Text wraps within container; no horizontal scrollbar appears; layout intact across breakpoints.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_056</t>
-  </si>
-  <si>
-    <t>Empty Videos list shows placeholder copy</t>
-  </si>
-  <si>
-    <t>Strapi returns no videos</t>
-  </si>
-  <si>
-    <t>1. Open Videos page</t>
-  </si>
-  <si>
-    <t>Empty-state copy (e.g., "No videos available yet"); section heading still renders; no broken layout.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_058</t>
-  </si>
-  <si>
-    <t>Video embed plays without leaking CP session credentials</t>
-  </si>
-  <si>
-    <t>Video uses third-party embed (YouTube/Vimeo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click and play a video
-2. Inspect outbound requests in network tab</t>
-  </si>
-  <si>
-    <t>Requests go directly to third-party host; no XR JWT / cookies forwarded; embed renders inside iframe sandbox.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_060</t>
-  </si>
-  <si>
-    <t>Videos page is identical for Master CP and Member CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Login as M, list videos
-2. Login as N, list videos</t>
-  </si>
-  <si>
-    <t>Same video list both times — no per-CP scoping in Strapi (CP-PI-003). Confirms no project-assignment table on CP side.</t>
+    <t>CP_PROJ_053</t>
+  </si>
+  <si>
+    <t>Key Points HTML content uses safe rendering (NOT dangerouslySetInnerHTML)</t>
+  </si>
+  <si>
+    <t>Strapi key-point contains `&lt;script&gt;alert(1)&lt;/script&gt;` string</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Key Points page
+2. Inspect DOM</t>
+  </si>
+  <si>
+    <t>Script tag rendered as escaped text (NOT executed). If it executes → file as XSS gap analogous to CP_PROJ_033 / CP-PI-004. Verify keyPoints uses safe text rendering.</t>
   </si>
   <si>
     <t>CP_PROJ_061</t>
@@ -4254,348 +4599,6 @@
   </si>
   <si>
     <t>PDF downloads/renders directly from Strapi without auth — raw asset URL with no expiry / signature (CP-PI-005). Document risk; confirm with security if acceptable.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_033</t>
-  </si>
-  <si>
-    <t>`information` field XSS via Strapi WYSIWYG (potential)</t>
-  </si>
-  <si>
-    <t>Admin can write to Strapi `information` field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Insert `&lt;script&gt;alert(1)&lt;/script&gt;` via Strapi admin
-2. Open `/project1/projectInfo`</t>
-  </si>
-  <si>
-    <t>Script executes in CP browser — frontend uses `dangerouslySetInnerHTML` without sanitization (CP-PI-004, projectInfo.jsx:14). Trust boundary depends entirely on Strapi authoring controls. Document as security gap.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_035</t>
-  </si>
-  <si>
-    <t>Single-newline whitespace in `information` collapses (UX gap)</t>
-  </si>
-  <si>
-    <t>Author writes content with single newlines between sentences</t>
-  </si>
-  <si>
-    <t>1. Render Project Info page</t>
-  </si>
-  <si>
-    <t>Single `\n` is dropped; only `\n\n` converted to `&lt;br /&gt;&lt;br /&gt;` (CP-PI-009, projectInfo.jsx:14). Authors must use double-newline.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_037</t>
-  </si>
-  <si>
-    <t>About section sources `information` field directly from Strapi</t>
-  </si>
-  <si>
-    <t>CP logged in; About page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to `/project1/about`
-2. Inspect network requests</t>
-  </si>
-  <si>
-    <t>A `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` is fired directly from the CP browser; About content renders from `data.attributes.information` field (CP-PI-002, Urls.js:7). No XR backend call for project content.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_040</t>
-  </si>
-  <si>
-    <t>About section shows empty placeholder when `information` is null</t>
-  </si>
-  <si>
-    <t>Strapi `information` field is null or empty string</t>
-  </si>
-  <si>
-    <t>1. Open About page</t>
-  </si>
-  <si>
-    <t>Page renders heading; body shows empty placeholder or no content paragraph (NOT a JS error or broken layout).</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  BUSINESS RULE TESTS  (1)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_047</t>
-  </si>
-  <si>
-    <t>Amenities returns DRAFT entries via populate=deep (publish gating bug)</t>
-  </si>
-  <si>
-    <t>Admin creates an amenity in Strapi but does NOT publish it</t>
-  </si>
-  <si>
-    <t>1. Open Amenities page in CP</t>
-  </si>
-  <si>
-    <t>Verify whether draft amenity appears. `populate=deep` may include DRAFT + PUBLISHED unless `publicationState=live` is passed (CP-PI-008, QA-Risk-14). If DRAFT visible → document as bug.</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  INTEGRATION TESTS  (15)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_025</t>
-  </si>
-  <si>
-    <t>Content reflects latest Strapi publish</t>
-  </si>
-  <si>
-    <t>Admin has published an update in Strapi CMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open the affected section in CP portal
-2. Hard refresh</t>
-  </si>
-  <si>
-    <t>Updated content is visible reflecting the latest Strapi publish</t>
-  </si>
-  <si>
-    <t>CP_PROJ_030</t>
-  </si>
-  <si>
-    <t>Frontend fetches Strapi directly (no XR proxy)</t>
-  </si>
-  <si>
-    <t>CP logged in, network tab open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/about`
-2. Inspect network requests</t>
-  </si>
-  <si>
-    <t>Direct `GET &lt;BaseURL&gt;/api/projects/1?populate=deep` to Strapi host. NO request to XR backend `/api/v1/*` for project content (Urls.js:7).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_032</t>
-  </si>
-  <si>
-    <t>Strapi outage breaks CP project pages silently</t>
-  </si>
-  <si>
-    <t>Block Strapi URL in browser</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/about`</t>
-  </si>
-  <si>
-    <t>Frontend fails to render — no XR-side circuit breaker / cache (CP-PI-007). UI may white-screen. Document accessibility implications.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_034</t>
-  </si>
-  <si>
-    <t>Brochure URL is unsigned Strapi asset (shareable externally)</t>
-  </si>
-  <si>
-    <t>Project info page open with brochure published</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Copy brochure URL from `data.brochure.data.attributes.url`
-2. Open in incognito (no CP session)</t>
-  </si>
-  <si>
-    <t>PDF downloads without auth — raw Strapi URL, no presigned/expiry (CP-PI-005). Confirm with security if acceptable.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_041</t>
-  </si>
-  <si>
-    <t>About reflects latest Strapi publish without hard refresh delay</t>
-  </si>
-  <si>
-    <t>Admin updates `information` in Strapi and clicks Publish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. CP performs hard refresh on `/project1/about` (Ctrl+Shift+R)
-2. Read content</t>
-  </si>
-  <si>
-    <t>Updated content appears immediately — no XR-side ISR/cache (CP-PI-007). Browser fetch hits Strapi live each load.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_043</t>
-  </si>
-  <si>
-    <t>Amenities list sourced from Strapi `amenities` relation</t>
-  </si>
-  <si>
-    <t>Amenities page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/amenities`
-2. Inspect Strapi response</t>
-  </si>
-  <si>
-    <t>Amenity items rendered from `data.attributes.amenities.data[].attributes` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). Each item shows name + icon URL.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_044</t>
-  </si>
-  <si>
-    <t>Amenity icons load from Strapi asset URLs without 404s</t>
-  </si>
-  <si>
-    <t>Strapi amenities have published icon assets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render Amenities list
-2. Observe icon image requests in network tab</t>
-  </si>
-  <si>
-    <t>Every icon URL (raw Strapi `attributes.url`) returns 200; no broken-image placeholders; unsigned URLs cacheable (CP-PI-005).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_046</t>
-  </si>
-  <si>
-    <t>Strapi outage breaks Amenities section silently</t>
-  </si>
-  <si>
-    <t>Block Strapi host in browser DevTools</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/amenities`</t>
-  </si>
-  <si>
-    <t>Frontend has NO XR-side fallback — section either white-screens or shows error boundary (CP-PI-007). No cached version served by XR backend. Document accessibility/UX gap.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_049</t>
-  </si>
-  <si>
-    <t>Key Points sourced from Strapi `keyPoints` field</t>
-  </si>
-  <si>
-    <t>Key Points page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/keyPoints`
-2. Inspect Strapi response</t>
-  </si>
-  <si>
-    <t>List items rendered from `data.attributes.keyPoints` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). No XR backend route involved.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_050</t>
-  </si>
-  <si>
-    <t>Key Points renders ordered list with correct sequence from Strapi</t>
-  </si>
-  <si>
-    <t>Strapi has 5 key-point entries in defined order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render Key Points page
-2. Read items top → bottom</t>
-  </si>
-  <si>
-    <t>Items render in the same order as the Strapi array; no client-side re-sort; numbering / bullets follow source ordering.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_054</t>
-  </si>
-  <si>
-    <t>Key Points reflects latest Strapi publish after hard refresh</t>
-  </si>
-  <si>
-    <t>Admin publishes a new key-point in Strapi</t>
-  </si>
-  <si>
-    <t>1. CP performs Ctrl+Shift+R on `/project1/keyPoints`</t>
-  </si>
-  <si>
-    <t>New point appears immediately — no XR-side cache (CP-PI-007). Browser request hits Strapi live.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_055</t>
-  </si>
-  <si>
-    <t>Videos list sourced from Strapi `videos` relation</t>
-  </si>
-  <si>
-    <t>Videos page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/videos`
-2. Inspect Strapi response</t>
-  </si>
-  <si>
-    <t>Items rendered from `data.attributes.videos.data[]` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). Each item supplies a video URL/embed code + thumbnail.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_057</t>
-  </si>
-  <si>
-    <t>Video thumbnails load from Strapi asset URLs</t>
-  </si>
-  <si>
-    <t>At least 2 published videos in Strapi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render Videos page
-2. Inspect each `&lt;img&gt;` request</t>
-  </si>
-  <si>
-    <t>Thumbnail URLs (raw Strapi asset) return 200; no 404s; unsigned URLs cacheable; same external-shareable trait as brochure assets (CP-PI-005).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_063</t>
-  </si>
-  <si>
-    <t>Strapi DRAFT entries should not leak via `populate=deep`</t>
-  </si>
-  <si>
-    <t>Admin creates a DRAFT entry in any populated relation (gallery/videos/keyPoints/amenities) without publishing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/&lt;section&gt;` as CP
-2. Compare visible items vs Strapi admin</t>
-  </si>
-  <si>
-    <t>Only PUBLISHED entries should render. If DRAFT appears → file as bug (CP-PI-008, QA-Risk-14). Fix is to add `publicationState=live` to Strapi URL.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_064</t>
-  </si>
-  <si>
-    <t>Hard refresh always fetches latest Strapi state (no XR cache)</t>
-  </si>
-  <si>
-    <t>Admin publishes a content edit in Strapi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. CP triggers Ctrl+Shift+R on any project section
-2. Inspect network requests</t>
-  </si>
-  <si>
-    <t>A fresh `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` is fired (no 304 / cache-hit on XR side); response reflects newly published content (CP-PI-007). Confirms no XR-side ISR / caching.</t>
-  </si>
-  <si>
-    <t>CORRECTION — There is NO XR backend endpoint for CP project info</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  NEGATIVE TESTS  (1)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_059</t>
-  </si>
-  <si>
-    <t>Broken/invalid video URL falls back gracefully</t>
-  </si>
-  <si>
-    <t>A Strapi video item has malformed URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Videos page
-2. Click the broken video</t>
-  </si>
-  <si>
-    <t>Embedded player shows its own error UI (or thumbnail with "Unavailable" overlay); page does not crash; other videos remain playable.</t>
   </si>
 </sst>
 </file>
@@ -13529,7 +13532,7 @@
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>1148</v>
+        <v>928</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -13543,25 +13546,25 @@
     </row>
     <row r="4" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>1149</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>1150</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="16" t="s">
+        <v>1150</v>
+      </c>
+      <c r="E4" s="16" t="s">
         <v>1151</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="16" t="s">
         <v>1152</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="16" t="s">
         <v>1153</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>1154</v>
       </c>
       <c r="H4" s="16" t="s">
         <v>28</v>
@@ -13575,25 +13578,25 @@
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="16" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E5" s="16" t="s">
         <v>1156</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="F5" s="16" t="s">
         <v>1157</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="G5" s="16" t="s">
         <v>1158</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>1159</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>28</v>
@@ -13607,25 +13610,25 @@
     </row>
     <row r="6" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>44</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>305</v>
       </c>
       <c r="F6" s="13" t="s">
+        <v>1161</v>
+      </c>
+      <c r="G6" s="13" t="s">
         <v>1162</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>1163</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>28</v>
@@ -13639,25 +13642,25 @@
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="E7" s="16" t="s">
         <v>305</v>
       </c>
       <c r="F7" s="16" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>1166</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>1167</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>28</v>
@@ -13671,25 +13674,25 @@
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="E8" s="16" t="s">
         <v>305</v>
       </c>
       <c r="F8" s="16" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G8" s="16" t="s">
         <v>1170</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>1171</v>
       </c>
       <c r="H8" s="16" t="s">
         <v>28</v>
@@ -13703,25 +13706,25 @@
     </row>
     <row r="9" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>44</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>305</v>
       </c>
       <c r="F9" s="13" t="s">
+        <v>1173</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>1174</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>1175</v>
       </c>
       <c r="H9" s="13" t="s">
         <v>28</v>
@@ -13735,25 +13738,25 @@
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>44</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>305</v>
       </c>
       <c r="F10" s="19" t="s">
+        <v>1177</v>
+      </c>
+      <c r="G10" s="19" t="s">
         <v>1178</v>
-      </c>
-      <c r="G10" s="19" t="s">
-        <v>1179</v>
       </c>
       <c r="H10" s="19" t="s">
         <v>28</v>
@@ -13767,25 +13770,25 @@
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>305</v>
       </c>
       <c r="F11" s="16" t="s">
+        <v>1181</v>
+      </c>
+      <c r="G11" s="16" t="s">
         <v>1182</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>1183</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>28</v>
@@ -13799,10 +13802,10 @@
     </row>
     <row r="12" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B12" s="16" t="s">
         <v>1184</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>1150</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>44</v>
@@ -13811,13 +13814,13 @@
         <v>1185</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>852</v>
+        <v>1186</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>28</v>
@@ -13831,25 +13834,25 @@
     </row>
     <row r="13" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="H13" s="16" t="s">
         <v>28</v>
@@ -13862,90 +13865,90 @@
       </c>
     </row>
     <row r="14" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>1194</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C14" s="14" t="s">
+      <c r="A14" s="18" t="s">
+        <v>1195</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>1190</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>1195</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>1191</v>
-      </c>
-      <c r="F14" s="13" t="s">
+      <c r="D14" s="19" t="s">
         <v>1196</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="E14" s="19" t="s">
         <v>1197</v>
       </c>
-      <c r="H14" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="I14" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>17</v>
+      <c r="F14" s="19" t="s">
+        <v>1198</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>1199</v>
+      </c>
+      <c r="H14" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="19" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="18" t="s">
-        <v>1198</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C15" s="20" t="s">
+      <c r="A15" s="15" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C15" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="19" t="s">
-        <v>1200</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>1201</v>
-      </c>
-      <c r="F15" s="19" t="s">
+      <c r="D15" s="16" t="s">
         <v>1202</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="E15" s="16" t="s">
         <v>1203</v>
       </c>
-      <c r="H15" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J15" s="19" t="s">
-        <v>62</v>
+      <c r="F15" s="16" t="s">
+        <v>1204</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>1205</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J15" s="16" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="16" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>1204</v>
+        <v>1206</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>1205</v>
+        <v>1207</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>1207</v>
+        <v>1209</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>1208</v>
+        <v>1210</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>1209</v>
+        <v>1211</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>28</v>
@@ -13959,25 +13962,25 @@
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>1210</v>
+        <v>1212</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>1211</v>
+        <v>1213</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>1212</v>
+        <v>1214</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>1213</v>
+        <v>1215</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>1214</v>
+        <v>1216</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>1215</v>
+        <v>1217</v>
       </c>
       <c r="H17" s="16" t="s">
         <v>28</v>
@@ -13990,58 +13993,58 @@
       </c>
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
-        <v>1216</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>1211</v>
-      </c>
-      <c r="C18" s="20" t="s">
+      <c r="A18" s="15" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C18" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="19" t="s">
-        <v>1217</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>1213</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G18" s="19" t="s">
-        <v>1219</v>
-      </c>
-      <c r="H18" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J18" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D18" s="16" t="s">
+        <v>1220</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>1221</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>1222</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>1223</v>
+      </c>
+      <c r="H18" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J18" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
-        <v>1220</v>
+        <v>1224</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>1211</v>
+        <v>81</v>
       </c>
       <c r="C19" s="20" t="s">
         <v>44</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>1221</v>
+        <v>1225</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>1222</v>
+        <v>1226</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>1223</v>
+        <v>1227</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>1224</v>
+        <v>1228</v>
       </c>
       <c r="H19" s="19" t="s">
         <v>28</v>
@@ -14050,44 +14053,62 @@
         <v>28</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
-        <v>1225</v>
-      </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="18" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>1230</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>1231</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>1232</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>1233</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J20" s="19" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>80</v>
+        <v>1234</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>81</v>
+        <v>1213</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>83</v>
+        <v>1235</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>28</v>
+        <v>1236</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>28</v>
+        <v>1237</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>28</v>
+        <v>1238</v>
       </c>
       <c r="H21" s="19" t="s">
         <v>28</v>
@@ -14096,62 +14117,44 @@
         <v>28</v>
       </c>
       <c r="J21" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>1226</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>1227</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>1228</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>1229</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>1230</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>1231</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J22" s="16" t="s">
-        <v>10</v>
-      </c>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>1232</v>
+        <v>80</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>1227</v>
+        <v>81</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>82</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>1233</v>
+        <v>83</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>1234</v>
+        <v>28</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>1235</v>
+        <v>28</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>1236</v>
+        <v>28</v>
       </c>
       <c r="H23" s="19" t="s">
         <v>28</v>
@@ -14160,126 +14163,126 @@
         <v>28</v>
       </c>
       <c r="J23" s="19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>1241</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>1242</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>1243</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>1244</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J24" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>1247</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>1248</v>
+      </c>
+      <c r="G25" s="19" t="s">
+        <v>1249</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I25" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J25" s="19" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="24" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
-        <v>1237</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>1227</v>
-      </c>
-      <c r="C24" s="20" t="s">
+    <row r="26" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="18" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C26" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="D24" s="19" t="s">
-        <v>1238</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>1239</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>1240</v>
-      </c>
-      <c r="G24" s="19" t="s">
-        <v>1241</v>
-      </c>
-      <c r="H24" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I24" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J24" s="19" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>1242</v>
-      </c>
-      <c r="B25" s="16" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C25" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>1243</v>
-      </c>
-      <c r="E25" s="16" t="s">
-        <v>1244</v>
-      </c>
-      <c r="F25" s="16" t="s">
-        <v>1245</v>
-      </c>
-      <c r="G25" s="16" t="s">
-        <v>1246</v>
-      </c>
-      <c r="H25" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I25" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J25" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>1247</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>1205</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>1248</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>1207</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>1249</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>1250</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="J26" s="13" t="s">
-        <v>17</v>
+      <c r="D26" s="19" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>1253</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>1254</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>1255</v>
+      </c>
+      <c r="H26" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J26" s="19" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="27" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>1251</v>
+        <v>1256</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>1205</v>
+        <v>1184</v>
       </c>
       <c r="C27" s="17" t="s">
         <v>82</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>1252</v>
+        <v>1257</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>1253</v>
+        <v>1258</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>1254</v>
+        <v>1259</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>1255</v>
+        <v>1260</v>
       </c>
       <c r="H27" s="16" t="s">
         <v>28</v>
@@ -14292,122 +14295,104 @@
       </c>
     </row>
     <row r="28" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>1256</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C28" s="17" t="s">
+      <c r="A28" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="D28" s="16" t="s">
-        <v>1258</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>1259</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>1260</v>
-      </c>
-      <c r="G28" s="16" t="s">
+      <c r="D28" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="H28" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I28" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J28" s="19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
         <v>1261</v>
       </c>
-      <c r="H28" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J28" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="18" t="s">
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
+    </row>
+    <row r="30" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
         <v>1262</v>
       </c>
-      <c r="B29" s="19" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D29" s="19" t="s">
+      <c r="B30" s="13" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" s="13" t="s">
         <v>1263</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E30" s="13" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F30" s="13" t="s">
         <v>1264</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="G30" s="13" t="s">
         <v>1265</v>
       </c>
-      <c r="G29" s="19" t="s">
-        <v>1266</v>
-      </c>
-      <c r="H29" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I29" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J29" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="18" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C30" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E30" s="19" t="s">
-        <v>1270</v>
-      </c>
-      <c r="F30" s="19" t="s">
-        <v>1271</v>
-      </c>
-      <c r="G30" s="19" t="s">
-        <v>1272</v>
-      </c>
-      <c r="H30" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I30" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J30" s="19" t="s">
-        <v>62</v>
+      <c r="H30" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="31" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
-        <v>1273</v>
+        <v>1266</v>
       </c>
       <c r="B31" s="19" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>1267</v>
+      </c>
+      <c r="E31" s="19" t="s">
         <v>1268</v>
       </c>
-      <c r="C31" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>1274</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>1275</v>
-      </c>
       <c r="F31" s="19" t="s">
-        <v>1276</v>
+        <v>1269</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>1277</v>
+        <v>1270</v>
       </c>
       <c r="H31" s="19" t="s">
         <v>28</v>
@@ -14419,123 +14404,123 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="18" t="s">
+    <row r="32" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>1272</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>1273</v>
+      </c>
+      <c r="G32" s="13" t="s">
+        <v>1274</v>
+      </c>
+      <c r="H32" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="I32" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="18" t="s">
+        <v>1275</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>1276</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>1215</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>1277</v>
+      </c>
+      <c r="G33" s="19" t="s">
         <v>1278</v>
       </c>
-      <c r="B32" s="19" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D32" s="19" t="s">
+      <c r="H33" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I33" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="18" t="s">
         <v>1279</v>
       </c>
-      <c r="E32" s="19" t="s">
+      <c r="B34" s="19" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C34" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D34" s="19" t="s">
         <v>1280</v>
       </c>
-      <c r="F32" s="19" t="s">
+      <c r="E34" s="19" t="s">
         <v>1281</v>
       </c>
-      <c r="G32" s="19" t="s">
+      <c r="F34" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="H32" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I32" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J32" s="19" t="s">
+      <c r="G34" s="19" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J34" s="19" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
-        <v>1283</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>1205</v>
-      </c>
-      <c r="C33" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D33" s="16" t="s">
+    <row r="35" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="18" t="s">
         <v>1284</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="B35" s="19" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C35" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D35" s="19" t="s">
         <v>1285</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="E35" s="19" t="s">
         <v>1286</v>
       </c>
-      <c r="G33" s="16" t="s">
+      <c r="F35" s="19" t="s">
         <v>1287</v>
       </c>
-      <c r="H33" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I33" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J33" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="34" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="18" t="s">
+      <c r="G35" s="19" t="s">
         <v>1288</v>
-      </c>
-      <c r="B34" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D34" s="19" t="s">
-        <v>1289</v>
-      </c>
-      <c r="E34" s="19" t="s">
-        <v>1290</v>
-      </c>
-      <c r="F34" s="19" t="s">
-        <v>1291</v>
-      </c>
-      <c r="G34" s="19" t="s">
-        <v>1292</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I34" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J34" s="19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="35" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="18" t="s">
-        <v>1293</v>
-      </c>
-      <c r="B35" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C35" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" s="19" t="s">
-        <v>1294</v>
-      </c>
-      <c r="E35" s="19" t="s">
-        <v>1295</v>
-      </c>
-      <c r="F35" s="19" t="s">
-        <v>1296</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>1297</v>
       </c>
       <c r="H35" s="19" t="s">
         <v>28</v>
@@ -14547,27 +14532,27 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
-        <v>1298</v>
+        <v>1289</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>1189</v>
+        <v>81</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>82</v>
+        <v>160</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>1299</v>
+        <v>1290</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>1300</v>
+        <v>1291</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>1301</v>
+        <v>1292</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>1302</v>
+        <v>1293</v>
       </c>
       <c r="H36" s="19" t="s">
         <v>28</v>
@@ -14576,30 +14561,30 @@
         <v>28</v>
       </c>
       <c r="J36" s="19" t="s">
-        <v>247</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
-        <v>1303</v>
+        <v>1294</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>1189</v>
+        <v>1184</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>82</v>
+        <v>160</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>1304</v>
+        <v>1295</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>1305</v>
+        <v>1296</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>1306</v>
+        <v>1297</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>1307</v>
+        <v>1298</v>
       </c>
       <c r="H37" s="19" t="s">
         <v>28</v>
@@ -14611,187 +14596,169 @@
         <v>247</v>
       </c>
     </row>
-    <row r="38" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>1300</v>
+      </c>
+      <c r="E38" s="19" t="s">
+        <v>1286</v>
+      </c>
+      <c r="F38" s="19" t="s">
+        <v>1301</v>
+      </c>
+      <c r="G38" s="19" t="s">
+        <v>1302</v>
+      </c>
+      <c r="H38" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I38" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J38" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="18" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>1304</v>
+      </c>
+      <c r="E39" s="19" t="s">
+        <v>1286</v>
+      </c>
+      <c r="F39" s="19" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G39" s="19" t="s">
+        <v>1306</v>
+      </c>
+      <c r="H39" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I39" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J39" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="11" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="11"/>
+    </row>
+    <row r="41" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="15" t="s">
         <v>1308</v>
       </c>
-      <c r="B38" s="19" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C38" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D38" s="19" t="s">
+      <c r="B41" s="16" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D41" s="16" t="s">
         <v>1309</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="E41" s="16" t="s">
         <v>1310</v>
       </c>
-      <c r="F38" s="19" t="s">
+      <c r="F41" s="16" t="s">
         <v>1311</v>
       </c>
-      <c r="G38" s="19" t="s">
+      <c r="G41" s="16" t="s">
         <v>1312</v>
       </c>
-      <c r="H38" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I38" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J38" s="19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="39" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
+      <c r="H41" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I41" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J41" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="15" t="s">
         <v>1313</v>
       </c>
-      <c r="B39" s="16" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C39" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D39" s="16" t="s">
+      <c r="B42" s="16" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D42" s="16" t="s">
         <v>1314</v>
       </c>
-      <c r="E39" s="16" t="s">
+      <c r="E42" s="16" t="s">
         <v>1315</v>
       </c>
-      <c r="F39" s="16" t="s">
+      <c r="F42" s="16" t="s">
         <v>1316</v>
       </c>
-      <c r="G39" s="16" t="s">
+      <c r="G42" s="16" t="s">
         <v>1317</v>
       </c>
-      <c r="H39" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I39" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J39" s="16" t="s">
+      <c r="H42" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J42" s="16" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="40" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="18" t="s">
-        <v>1318</v>
-      </c>
-      <c r="B40" s="19" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C40" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D40" s="19" t="s">
-        <v>1319</v>
-      </c>
-      <c r="E40" s="19" t="s">
-        <v>1320</v>
-      </c>
-      <c r="F40" s="19" t="s">
-        <v>1321</v>
-      </c>
-      <c r="G40" s="19" t="s">
-        <v>1322</v>
-      </c>
-      <c r="H40" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I40" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J40" s="19" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="41" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="18" t="s">
-        <v>1323</v>
-      </c>
-      <c r="B41" s="19" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C41" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D41" s="19" t="s">
-        <v>1324</v>
-      </c>
-      <c r="E41" s="19" t="s">
-        <v>1280</v>
-      </c>
-      <c r="F41" s="19" t="s">
-        <v>1325</v>
-      </c>
-      <c r="G41" s="19" t="s">
-        <v>1326</v>
-      </c>
-      <c r="H41" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I41" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J41" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="42" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="18" t="s">
-        <v>1327</v>
-      </c>
-      <c r="B42" s="19" t="s">
-        <v>1211</v>
-      </c>
-      <c r="C42" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>1328</v>
-      </c>
-      <c r="E42" s="19" t="s">
-        <v>1329</v>
-      </c>
-      <c r="F42" s="19" t="s">
-        <v>1330</v>
-      </c>
-      <c r="G42" s="19" t="s">
-        <v>1331</v>
-      </c>
-      <c r="H42" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I42" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J42" s="19" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="43" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="18" t="s">
-        <v>1332</v>
+        <v>1318</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>1211</v>
+        <v>1184</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>82</v>
+        <v>208</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>1333</v>
+        <v>1319</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>1334</v>
+        <v>1320</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>1335</v>
+        <v>1321</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>1336</v>
+        <v>1322</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>28</v>
@@ -14803,297 +14770,315 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="18" t="s">
+    <row r="44" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="15" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B44" s="16" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C44" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>1325</v>
+      </c>
+      <c r="F44" s="16" t="s">
+        <v>1326</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>1327</v>
+      </c>
+      <c r="H44" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I44" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J44" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="15" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D45" s="16" t="s">
+        <v>1329</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>1330</v>
+      </c>
+      <c r="F45" s="16" t="s">
+        <v>1331</v>
+      </c>
+      <c r="G45" s="16" t="s">
+        <v>1332</v>
+      </c>
+      <c r="H45" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I45" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J45" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="15" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B46" s="16" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C46" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>1334</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>1335</v>
+      </c>
+      <c r="F46" s="16" t="s">
+        <v>1336</v>
+      </c>
+      <c r="G46" s="16" t="s">
         <v>1337</v>
       </c>
-      <c r="B44" s="19" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C44" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D44" s="19" t="s">
+      <c r="H46" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I46" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J46" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="18" t="s">
         <v>1338</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="B47" s="19" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="D47" s="19" t="s">
         <v>1339</v>
       </c>
-      <c r="F44" s="19" t="s">
+      <c r="E47" s="19" t="s">
         <v>1340</v>
       </c>
-      <c r="G44" s="19" t="s">
+      <c r="F47" s="19" t="s">
         <v>1341</v>
       </c>
-      <c r="H44" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I44" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J44" s="19" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="45" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="18" t="s">
+      <c r="G47" s="19" t="s">
         <v>1342</v>
       </c>
-      <c r="B45" s="19" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C45" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D45" s="19" t="s">
+      <c r="H47" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I47" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J47" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="18" t="s">
         <v>1343</v>
       </c>
-      <c r="E45" s="19" t="s">
+      <c r="B48" s="19" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="D48" s="19" t="s">
         <v>1344</v>
       </c>
-      <c r="F45" s="19" t="s">
+      <c r="E48" s="19" t="s">
         <v>1345</v>
       </c>
-      <c r="G45" s="19" t="s">
+      <c r="F48" s="19" t="s">
         <v>1346</v>
       </c>
-      <c r="H45" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I45" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J45" s="19" t="s">
-        <v>1067</v>
-      </c>
-    </row>
-    <row r="46" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="18" t="s">
+      <c r="G48" s="19" t="s">
         <v>1347</v>
       </c>
-      <c r="B46" s="19" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C46" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D46" s="19" t="s">
+      <c r="H48" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I48" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J48" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="15" t="s">
         <v>1348</v>
       </c>
-      <c r="E46" s="19" t="s">
-        <v>1280</v>
-      </c>
-      <c r="F46" s="19" t="s">
+      <c r="B49" s="16" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C49" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D49" s="16" t="s">
         <v>1349</v>
       </c>
-      <c r="G46" s="19" t="s">
+      <c r="E49" s="16" t="s">
         <v>1350</v>
       </c>
-      <c r="H46" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I46" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J46" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="47" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="15" t="s">
+      <c r="F49" s="16" t="s">
         <v>1351</v>
       </c>
-      <c r="B47" s="16" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C47" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="D47" s="16" t="s">
+      <c r="G49" s="16" t="s">
         <v>1352</v>
       </c>
-      <c r="E47" s="16" t="s">
+      <c r="H49" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I49" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J49" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" s="15" t="s">
         <v>1353</v>
       </c>
-      <c r="F47" s="16" t="s">
+      <c r="B50" s="16" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C50" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D50" s="16" t="s">
         <v>1354</v>
       </c>
-      <c r="G47" s="16" t="s">
+      <c r="E50" s="16" t="s">
         <v>1355</v>
       </c>
-      <c r="H47" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I47" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J47" s="16" t="s">
+      <c r="F50" s="16" t="s">
+        <v>1356</v>
+      </c>
+      <c r="G50" s="16" t="s">
+        <v>1357</v>
+      </c>
+      <c r="H50" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I50" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J50" s="16" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="48" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="18" t="s">
-        <v>1356</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D48" s="19" t="s">
-        <v>1357</v>
-      </c>
-      <c r="E48" s="19" t="s">
-        <v>1358</v>
-      </c>
-      <c r="F48" s="19" t="s">
-        <v>1359</v>
-      </c>
-      <c r="G48" s="19" t="s">
-        <v>1360</v>
-      </c>
-      <c r="H48" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I48" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J48" s="19" t="s">
-        <v>1067</v>
-      </c>
-    </row>
-    <row r="49" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="B49" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C49" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D49" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="F49" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="G49" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="H49" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I49" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J49" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="11" t="s">
-        <v>1031</v>
-      </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
-      <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="11"/>
-      <c r="J50" s="11"/>
     </row>
     <row r="51" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="18" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B51" s="19" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C51" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>1359</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>1360</v>
+      </c>
+      <c r="F51" s="19" t="s">
         <v>1361</v>
       </c>
-      <c r="B51" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C51" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="D51" s="19" t="s">
+      <c r="G51" s="19" t="s">
         <v>1362</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="H51" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I51" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J51" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" s="15" t="s">
         <v>1363</v>
       </c>
-      <c r="F51" s="19" t="s">
+      <c r="B52" s="16" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C52" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D52" s="16" t="s">
         <v>1364</v>
       </c>
-      <c r="G51" s="19" t="s">
+      <c r="E52" s="16" t="s">
         <v>1365</v>
       </c>
-      <c r="H51" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I51" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J51" s="19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="52" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" s="18" t="s">
+      <c r="F52" s="16" t="s">
         <v>1366</v>
       </c>
-      <c r="B52" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C52" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="D52" s="19" t="s">
+      <c r="G52" s="16" t="s">
         <v>1367</v>
       </c>
-      <c r="E52" s="19" t="s">
-        <v>1368</v>
-      </c>
-      <c r="F52" s="19" t="s">
-        <v>1369</v>
-      </c>
-      <c r="G52" s="19" t="s">
-        <v>1370</v>
-      </c>
-      <c r="H52" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I52" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J52" s="19" t="s">
-        <v>247</v>
+      <c r="H52" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I52" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52" s="16" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="53" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="15" t="s">
+        <v>1368</v>
+      </c>
+      <c r="B53" s="16" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C53" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D53" s="16" t="s">
+        <v>1369</v>
+      </c>
+      <c r="E53" s="16" t="s">
+        <v>1370</v>
+      </c>
+      <c r="F53" s="16" t="s">
         <v>1371</v>
       </c>
-      <c r="B53" s="16" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C53" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D53" s="16" t="s">
+      <c r="G53" s="16" t="s">
         <v>1372</v>
-      </c>
-      <c r="E53" s="16" t="s">
-        <v>1373</v>
-      </c>
-      <c r="F53" s="16" t="s">
-        <v>1374</v>
-      </c>
-      <c r="G53" s="16" t="s">
-        <v>1375</v>
       </c>
       <c r="H53" s="16" t="s">
         <v>28</v>
@@ -15105,27 +15090,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="18" t="s">
+        <v>1373</v>
+      </c>
+      <c r="B54" s="19" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C54" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="D54" s="19" t="s">
+        <v>1374</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>1375</v>
+      </c>
+      <c r="F54" s="19" t="s">
         <v>1376</v>
       </c>
-      <c r="B54" s="19" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C54" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="D54" s="19" t="s">
+      <c r="G54" s="19" t="s">
         <v>1377</v>
-      </c>
-      <c r="E54" s="19" t="s">
-        <v>1378</v>
-      </c>
-      <c r="F54" s="19" t="s">
-        <v>1379</v>
-      </c>
-      <c r="G54" s="19" t="s">
-        <v>1380</v>
       </c>
       <c r="H54" s="19" t="s">
         <v>28</v>
@@ -15137,41 +15122,59 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="11" t="s">
+    <row r="55" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="18" t="s">
+        <v>1378</v>
+      </c>
+      <c r="B55" s="19" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>1379</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>1380</v>
+      </c>
+      <c r="F55" s="19" t="s">
         <v>1381</v>
       </c>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="11"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="11"/>
-      <c r="J55" s="11"/>
-    </row>
-    <row r="56" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G55" s="19" t="s">
+        <v>1382</v>
+      </c>
+      <c r="H55" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I55" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J55" s="19" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="56" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>1199</v>
+        <v>1251</v>
       </c>
       <c r="C56" s="17" t="s">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="E56" s="16" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="G56" s="16" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
       <c r="H56" s="16" t="s">
         <v>28</v>
@@ -15183,73 +15186,73 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="11" t="s">
-        <v>1387</v>
-      </c>
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="11"/>
-      <c r="G57" s="11"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="11"/>
-      <c r="J57" s="11"/>
-    </row>
-    <row r="58" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" s="15" t="s">
+    <row r="57" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" s="18" t="s">
         <v>1388</v>
       </c>
-      <c r="B58" s="16" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C58" s="17" t="s">
+      <c r="B57" s="19" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C57" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="D58" s="16" t="s">
+      <c r="D57" s="19" t="s">
         <v>1389</v>
       </c>
-      <c r="E58" s="16" t="s">
+      <c r="E57" s="19" t="s">
         <v>1390</v>
       </c>
-      <c r="F58" s="16" t="s">
+      <c r="F57" s="19" t="s">
         <v>1391</v>
       </c>
-      <c r="G58" s="16" t="s">
+      <c r="G57" s="19" t="s">
         <v>1392</v>
       </c>
-      <c r="H58" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I58" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J58" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="59" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H57" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I57" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J57" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="11" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B58" s="11"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11"/>
+    </row>
+    <row r="59" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="15" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>1189</v>
+        <v>1207</v>
       </c>
       <c r="C59" s="17" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="D59" s="16" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
       <c r="H59" s="16" t="s">
         <v>28</v>
@@ -15261,27 +15264,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="18" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>1189</v>
+        <v>81</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="E60" s="19" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="F60" s="19" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
       <c r="G60" s="19" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="H60" s="19" t="s">
         <v>28</v>
@@ -15290,126 +15293,108 @@
         <v>28</v>
       </c>
       <c r="J60" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="61" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="61" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
-        <v>1403</v>
+        <v>801</v>
       </c>
       <c r="B61" s="19" t="s">
         <v>81</v>
       </c>
       <c r="C61" s="20" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="D61" s="19" t="s">
         <v>1404</v>
       </c>
       <c r="E61" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F61" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="G61" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="H61" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I61" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J61" s="19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="11" t="s">
         <v>1405</v>
       </c>
-      <c r="F61" s="19" t="s">
+      <c r="B62" s="11"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="11"/>
+      <c r="E62" s="11"/>
+      <c r="F62" s="11"/>
+      <c r="G62" s="11"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
+      <c r="J62" s="11"/>
+    </row>
+    <row r="63" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="18" t="s">
         <v>1406</v>
       </c>
-      <c r="G61" s="19" t="s">
+      <c r="B63" s="19" t="s">
+        <v>1190</v>
+      </c>
+      <c r="C63" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D63" s="19" t="s">
         <v>1407</v>
       </c>
-      <c r="H61" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I61" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J61" s="19" t="s">
-        <v>1067</v>
-      </c>
-    </row>
-    <row r="62" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="15" t="s">
+      <c r="E63" s="19" t="s">
         <v>1408</v>
       </c>
-      <c r="B62" s="16" t="s">
-        <v>1189</v>
-      </c>
-      <c r="C62" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="D62" s="16" t="s">
+      <c r="F63" s="19" t="s">
         <v>1409</v>
       </c>
-      <c r="E62" s="16" t="s">
+      <c r="G63" s="19" t="s">
         <v>1410</v>
       </c>
-      <c r="F62" s="16" t="s">
+      <c r="H63" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I63" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J63" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="64" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="18" t="s">
         <v>1411</v>
       </c>
-      <c r="G62" s="16" t="s">
+      <c r="B64" s="19" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C64" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D64" s="19" t="s">
         <v>1412</v>
       </c>
-      <c r="H62" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I62" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J62" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="63" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="15" t="s">
+      <c r="E64" s="19" t="s">
         <v>1413</v>
       </c>
-      <c r="B63" s="16" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C63" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="D63" s="16" t="s">
+      <c r="F64" s="19" t="s">
         <v>1414</v>
       </c>
-      <c r="E63" s="16" t="s">
+      <c r="G64" s="19" t="s">
         <v>1415</v>
-      </c>
-      <c r="F63" s="16" t="s">
-        <v>1416</v>
-      </c>
-      <c r="G63" s="16" t="s">
-        <v>1417</v>
-      </c>
-      <c r="H63" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I63" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J63" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="64" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" s="18" t="s">
-        <v>1418</v>
-      </c>
-      <c r="B64" s="19" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C64" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="D64" s="19" t="s">
-        <v>1419</v>
-      </c>
-      <c r="E64" s="19" t="s">
-        <v>1420</v>
-      </c>
-      <c r="F64" s="19" t="s">
-        <v>1421</v>
-      </c>
-      <c r="G64" s="19" t="s">
-        <v>1422</v>
       </c>
       <c r="H64" s="19" t="s">
         <v>28</v>
@@ -15423,341 +15408,359 @@
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
+        <v>1416</v>
+      </c>
+      <c r="B65" s="19" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C65" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D65" s="19" t="s">
+        <v>1417</v>
+      </c>
+      <c r="E65" s="19" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F65" s="19" t="s">
+        <v>1419</v>
+      </c>
+      <c r="G65" s="19" t="s">
+        <v>1420</v>
+      </c>
+      <c r="H65" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I65" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J65" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="66" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="18" t="s">
+        <v>1421</v>
+      </c>
+      <c r="B66" s="19" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C66" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D66" s="19" t="s">
+        <v>1422</v>
+      </c>
+      <c r="E66" s="19" t="s">
         <v>1423</v>
       </c>
-      <c r="B65" s="19" t="s">
-        <v>1199</v>
-      </c>
-      <c r="C65" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="D65" s="19" t="s">
+      <c r="F66" s="19" t="s">
         <v>1424</v>
       </c>
-      <c r="E65" s="19" t="s">
+      <c r="G66" s="19" t="s">
         <v>1425</v>
       </c>
-      <c r="F65" s="19" t="s">
+      <c r="H66" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I66" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J66" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="67" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="18" t="s">
         <v>1426</v>
       </c>
-      <c r="G65" s="19" t="s">
+      <c r="B67" s="19" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C67" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D67" s="19" t="s">
         <v>1427</v>
       </c>
-      <c r="H65" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I65" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J65" s="19" t="s">
+      <c r="E67" s="19" t="s">
+        <v>1428</v>
+      </c>
+      <c r="F67" s="19" t="s">
+        <v>1429</v>
+      </c>
+      <c r="G67" s="19" t="s">
+        <v>1430</v>
+      </c>
+      <c r="H67" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I67" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J67" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="68" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="18" t="s">
+        <v>1431</v>
+      </c>
+      <c r="B68" s="19" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C68" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="D68" s="19" t="s">
+        <v>1432</v>
+      </c>
+      <c r="E68" s="19" t="s">
+        <v>1433</v>
+      </c>
+      <c r="F68" s="19" t="s">
+        <v>1434</v>
+      </c>
+      <c r="G68" s="19" t="s">
+        <v>1435</v>
+      </c>
+      <c r="H68" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I68" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J68" s="19" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="66" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="15" t="s">
-        <v>1428</v>
-      </c>
-      <c r="B66" s="16" t="s">
-        <v>1211</v>
-      </c>
-      <c r="C66" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="D66" s="16" t="s">
-        <v>1429</v>
-      </c>
-      <c r="E66" s="16" t="s">
-        <v>1430</v>
-      </c>
-      <c r="F66" s="16" t="s">
-        <v>1431</v>
-      </c>
-      <c r="G66" s="16" t="s">
-        <v>1432</v>
-      </c>
-      <c r="H66" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I66" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J66" s="16" t="s">
+    <row r="69" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="11" t="s">
+        <v>1436</v>
+      </c>
+      <c r="B69" s="11"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="11"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="11"/>
+    </row>
+    <row r="70" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" s="15" t="s">
+        <v>1437</v>
+      </c>
+      <c r="B70" s="16" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C70" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="D70" s="16" t="s">
+        <v>1438</v>
+      </c>
+      <c r="E70" s="16" t="s">
+        <v>852</v>
+      </c>
+      <c r="F70" s="16" t="s">
+        <v>1439</v>
+      </c>
+      <c r="G70" s="16" t="s">
+        <v>1440</v>
+      </c>
+      <c r="H70" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I70" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J70" s="16" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="67" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A67" s="18" t="s">
-        <v>1433</v>
-      </c>
-      <c r="B67" s="19" t="s">
-        <v>1211</v>
-      </c>
-      <c r="C67" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="D67" s="19" t="s">
-        <v>1434</v>
-      </c>
-      <c r="E67" s="19" t="s">
-        <v>1435</v>
-      </c>
-      <c r="F67" s="19" t="s">
-        <v>1436</v>
-      </c>
-      <c r="G67" s="19" t="s">
-        <v>1437</v>
-      </c>
-      <c r="H67" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I67" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J67" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="68" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A68" s="15" t="s">
-        <v>1438</v>
-      </c>
-      <c r="B68" s="16" t="s">
-        <v>1211</v>
-      </c>
-      <c r="C68" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="D68" s="16" t="s">
-        <v>1439</v>
-      </c>
-      <c r="E68" s="16" t="s">
-        <v>1440</v>
-      </c>
-      <c r="F68" s="16" t="s">
+    <row r="71" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="18" t="s">
         <v>1441</v>
       </c>
-      <c r="G68" s="16" t="s">
+      <c r="B71" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C71" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="D71" s="19" t="s">
         <v>1442</v>
       </c>
-      <c r="H68" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I68" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J68" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="69" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A69" s="15" t="s">
+      <c r="E71" s="19" t="s">
         <v>1443</v>
       </c>
-      <c r="B69" s="16" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C69" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="D69" s="16" t="s">
+      <c r="F71" s="19" t="s">
         <v>1444</v>
       </c>
-      <c r="E69" s="16" t="s">
+      <c r="G71" s="19" t="s">
         <v>1445</v>
       </c>
-      <c r="F69" s="16" t="s">
-        <v>1446</v>
-      </c>
-      <c r="G69" s="16" t="s">
-        <v>1447</v>
-      </c>
-      <c r="H69" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I69" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J69" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="70" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" s="18" t="s">
-        <v>1448</v>
-      </c>
-      <c r="B70" s="19" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C70" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="D70" s="19" t="s">
-        <v>1449</v>
-      </c>
-      <c r="E70" s="19" t="s">
-        <v>1450</v>
-      </c>
-      <c r="F70" s="19" t="s">
-        <v>1451</v>
-      </c>
-      <c r="G70" s="19" t="s">
-        <v>1452</v>
-      </c>
-      <c r="H70" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I70" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J70" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="71" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A71" s="15" t="s">
-        <v>1453</v>
-      </c>
-      <c r="B71" s="16" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C71" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="D71" s="16" t="s">
-        <v>1454</v>
-      </c>
-      <c r="E71" s="16" t="s">
-        <v>1455</v>
-      </c>
-      <c r="F71" s="16" t="s">
-        <v>1456</v>
-      </c>
-      <c r="G71" s="16" t="s">
-        <v>1457</v>
-      </c>
-      <c r="H71" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I71" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="J71" s="16" t="s">
-        <v>10</v>
+      <c r="H71" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I71" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J71" s="19" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="72" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="18" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B72" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C72" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="D72" s="19" t="s">
+        <v>1447</v>
+      </c>
+      <c r="E72" s="19" t="s">
+        <v>1448</v>
+      </c>
+      <c r="F72" s="19" t="s">
+        <v>1449</v>
+      </c>
+      <c r="G72" s="19" t="s">
+        <v>1450</v>
+      </c>
+      <c r="H72" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I72" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J72" s="19" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="73" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" s="18" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B73" s="19" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C73" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="D73" s="19" t="s">
+        <v>1452</v>
+      </c>
+      <c r="E73" s="19" t="s">
+        <v>1453</v>
+      </c>
+      <c r="F73" s="19" t="s">
+        <v>1454</v>
+      </c>
+      <c r="G73" s="19" t="s">
+        <v>1455</v>
+      </c>
+      <c r="H73" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I73" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J73" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="74" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" s="18" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B74" s="19" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C74" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="D74" s="19" t="s">
+        <v>1457</v>
+      </c>
+      <c r="E74" s="19" t="s">
         <v>1458</v>
       </c>
-      <c r="B72" s="19" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C72" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="D72" s="19" t="s">
+      <c r="F74" s="19" t="s">
         <v>1459</v>
       </c>
-      <c r="E72" s="19" t="s">
+      <c r="G74" s="19" t="s">
         <v>1460</v>
       </c>
-      <c r="F72" s="19" t="s">
+      <c r="H74" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="I74" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J74" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="75" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" s="15" t="s">
         <v>1461</v>
       </c>
-      <c r="G72" s="19" t="s">
+      <c r="B75" s="16" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C75" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="D75" s="16" t="s">
         <v>1462</v>
       </c>
-      <c r="H72" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I72" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J72" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="73" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A73" s="11" t="s">
-        <v>678</v>
-      </c>
-      <c r="B73" s="11"/>
-      <c r="C73" s="11"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="11"/>
-      <c r="F73" s="11"/>
-      <c r="G73" s="11"/>
-      <c r="H73" s="11"/>
-      <c r="I73" s="11"/>
-      <c r="J73" s="11"/>
-    </row>
-    <row r="74" ht="40" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A74" s="18" t="s">
-        <v>801</v>
-      </c>
-      <c r="B74" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C74" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="D74" s="19" t="s">
+      <c r="E75" s="16" t="s">
         <v>1463</v>
       </c>
-      <c r="E74" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="F74" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="G74" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="H74" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I74" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J74" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="75" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" s="11" t="s">
+      <c r="F75" s="16" t="s">
         <v>1464</v>
       </c>
-      <c r="B75" s="11"/>
-      <c r="C75" s="11"/>
-      <c r="D75" s="11"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="11"/>
-      <c r="G75" s="11"/>
-      <c r="H75" s="11"/>
-      <c r="I75" s="11"/>
-      <c r="J75" s="11"/>
+      <c r="G75" s="16" t="s">
+        <v>1465</v>
+      </c>
+      <c r="H75" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I75" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J75" s="16" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="76" ht="44" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="18" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="B76" s="19" t="s">
-        <v>1257</v>
+        <v>1251</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>262</v>
       </c>
       <c r="D76" s="19" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
       <c r="E76" s="19" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="F76" s="19" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
       <c r="G76" s="19" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
       <c r="H76" s="19" t="s">
         <v>28</v>
@@ -15766,7 +15769,7 @@
         <v>28</v>
       </c>
       <c r="J76" s="19" t="s">
-        <v>62</v>
+        <v>1067</v>
       </c>
     </row>
   </sheetData>
@@ -15774,12 +15777,12 @@
   <mergeCells count="8">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A50:J50"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="A57:J57"/>
-    <mergeCell ref="A73:J73"/>
-    <mergeCell ref="A75:J75"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A40:J40"/>
+    <mergeCell ref="A58:J58"/>
+    <mergeCell ref="A62:J62"/>
+    <mergeCell ref="A69:J69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
chore(xlsx): clean stale/duplicate TCs — SM Callback, Buyer Unit Details, deprecated sheets
- SM Callback Requests: 268 → 86 rows (removed 172 TC_SMCB_* + non-unique SM_CB_*)
- Buyer Unit Details: 107 → 34 rows (removed 62 TC_UNIT_* + non-unique BYR_UNIT_*)
- Buyer Support Tickets sheet: removed (deprecated module, no BRD coverage)
- CP Project Information sheet: removed (deprecated module, no BRD coverage)
- Consolidated All Test Cases: 1110 → 1029 rows
- Added xlsx-cleanup-flags.md (362-line flagging report with wrong-ER documentation)
- Added cleanup-xlsx-stale-tcs.js (idempotent cleanup script, safe to re-run)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual-qa-repository/07-execution/TestCases-CPPortal.xlsx
+++ b/manual-qa-repository/07-execution/TestCases-CPPortal.xlsx
@@ -10,14 +10,13 @@
     <sheet sheetId="4" name="Customer Registration" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="KYC Assistance" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="JBP Submission" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Project Information" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7147" uniqueCount="2493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6119" uniqueCount="2170">
   <si>
     <t>CHANNEL PARTNER PORTAL — MASTER TEST CASE DOCUMENT</t>
   </si>
@@ -6689,1006 +6688,6 @@
   </si>
   <si>
     <t>`jbp-loaded.png` (CP side)</t>
-  </si>
-  <si>
-    <t>CHANNEL PARTNER PORTAL — Project Information Test Cases</t>
-  </si>
-  <si>
-    <t>CP_PROJ_001</t>
-  </si>
-  <si>
-    <t>Navigation and Access</t>
-  </si>
-  <si>
-    <t>Open Project Information from main nav</t>
-  </si>
-  <si>
-    <t>1. Click **Project** in the navigation menu</t>
-  </si>
-  <si>
-    <t>URL updates to `/project`; project overview page renders with section tabs</t>
-  </si>
-  <si>
-    <t>CP_PROJ_002</t>
-  </si>
-  <si>
-    <t>Section tabs are visible</t>
-  </si>
-  <si>
-    <t>Project overview open</t>
-  </si>
-  <si>
-    <t>1. Inspect tab bar</t>
-  </si>
-  <si>
-    <t>Tabs displayed: About, Gallery, Amenities, Documents, Key Points, Videos</t>
-  </si>
-  <si>
-    <t>CP_PROJ_003</t>
-  </si>
-  <si>
-    <t>Direct URL `/project1/about` loads About page</t>
-  </si>
-  <si>
-    <t>1. Navigate to `https://uat.xrportal.in/project1/about`</t>
-  </si>
-  <si>
-    <t>About page loads with project background, location, developer info</t>
-  </si>
-  <si>
-    <t>CP_PROJ_004</t>
-  </si>
-  <si>
-    <t>Direct URL `/project1/gallery` loads Gallery</t>
-  </si>
-  <si>
-    <t>1. Navigate to `/project1/gallery`</t>
-  </si>
-  <si>
-    <t>Gallery page loads with project photos</t>
-  </si>
-  <si>
-    <t>CP_PROJ_005</t>
-  </si>
-  <si>
-    <t>Direct URL `/project1/amenities` loads Amenities</t>
-  </si>
-  <si>
-    <t>1. Navigate to `/project1/amenities`</t>
-  </si>
-  <si>
-    <t>Amenities list renders with feature names and possible icons</t>
-  </si>
-  <si>
-    <t>CP_PROJ_006</t>
-  </si>
-  <si>
-    <t>Direct URL `/project1/documents` loads Documents</t>
-  </si>
-  <si>
-    <t>1. Navigate to `/project1/documents`</t>
-  </si>
-  <si>
-    <t>Documents page shows RERA, approvals, brochures with download links</t>
-  </si>
-  <si>
-    <t>CP_PROJ_007</t>
-  </si>
-  <si>
-    <t>Direct URL `/project1/keyPoints` loads Key Points</t>
-  </si>
-  <si>
-    <t>1. Navigate to `/project1/keyPoints`</t>
-  </si>
-  <si>
-    <t>Key selling points list renders</t>
-  </si>
-  <si>
-    <t>CP_PROJ_008</t>
-  </si>
-  <si>
-    <t>Direct URL `/project1/videos` loads Videos</t>
-  </si>
-  <si>
-    <t>1. Navigate to `/project1/videos`</t>
-  </si>
-  <si>
-    <t>Video gallery renders with embedded players or thumbnails</t>
-  </si>
-  <si>
-    <t>CP_PROJ_010</t>
-  </si>
-  <si>
-    <t>About Section</t>
-  </si>
-  <si>
-    <t>About displays project background text</t>
-  </si>
-  <si>
-    <t>About page open</t>
-  </si>
-  <si>
-    <t>1. Scroll through About content</t>
-  </si>
-  <si>
-    <t>Paragraphs describing project background, location, and developer are visible</t>
-  </si>
-  <si>
-    <t>CP_PROJ_012</t>
-  </si>
-  <si>
-    <t>Gallery</t>
-  </si>
-  <si>
-    <t>Gallery loads project photos in grid</t>
-  </si>
-  <si>
-    <t>Gallery page open</t>
-  </si>
-  <si>
-    <t>1. Scroll Gallery grid</t>
-  </si>
-  <si>
-    <t>Photos render in a grid layout; images load without 404s</t>
-  </si>
-  <si>
-    <t>CP_PROJ_013</t>
-  </si>
-  <si>
-    <t>Click a photo opens larger view</t>
-  </si>
-  <si>
-    <t>Gallery has at least one image</t>
-  </si>
-  <si>
-    <t>1. Click any thumbnail</t>
-  </si>
-  <si>
-    <t>Lightbox / modal opens displaying the full-size image with close control</t>
-  </si>
-  <si>
-    <t>CP_PROJ_015</t>
-  </si>
-  <si>
-    <t>Amenities</t>
-  </si>
-  <si>
-    <t>Amenities list renders with names</t>
-  </si>
-  <si>
-    <t>Amenities page open</t>
-  </si>
-  <si>
-    <t>1. Read items in the amenities list</t>
-  </si>
-  <si>
-    <t>Amenity names displayed; categories or icons present per Strapi configuration</t>
-  </si>
-  <si>
-    <t>CP_PROJ_017</t>
-  </si>
-  <si>
-    <t>Documents</t>
-  </si>
-  <si>
-    <t>RERA document is listed</t>
-  </si>
-  <si>
-    <t>Documents page open</t>
-  </si>
-  <si>
-    <t>1. Scan the document list</t>
-  </si>
-  <si>
-    <t>At least one entry labelled RERA Registration is present</t>
-  </si>
-  <si>
-    <t>CP_PROJ_020</t>
-  </si>
-  <si>
-    <t>Key Points</t>
-  </si>
-  <si>
-    <t>Key Points list is displayed</t>
-  </si>
-  <si>
-    <t>Key Points page open</t>
-  </si>
-  <si>
-    <t>1. Scroll list</t>
-  </si>
-  <si>
-    <t>Bullet/numbered list of key selling points renders as content</t>
-  </si>
-  <si>
-    <t>CP_PROJ_022</t>
-  </si>
-  <si>
-    <t>Videos</t>
-  </si>
-  <si>
-    <t>Videos page lists video thumbnails</t>
-  </si>
-  <si>
-    <t>Videos page open</t>
-  </si>
-  <si>
-    <t>1. Scroll list of videos</t>
-  </si>
-  <si>
-    <t>Video thumbnails or embeds render</t>
-  </si>
-  <si>
-    <t>CP_PROJ_035</t>
-  </si>
-  <si>
-    <t>Single-newline whitespace in `information` collapses (UX gap)</t>
-  </si>
-  <si>
-    <t>Author writes content with single newlines between sentences</t>
-  </si>
-  <si>
-    <t>1. Render Project Info page</t>
-  </si>
-  <si>
-    <t>Single `\n` is dropped; only `\n\n` converted to `&lt;br /&gt;&lt;br /&gt;` (CP-PI-009, projectInfo.jsx:14). Authors must use double-newline.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_038</t>
-  </si>
-  <si>
-    <t>About content renders double-newline as paragraph break</t>
-  </si>
-  <si>
-    <t>Strapi `information` field contains `Para A\n\nPara B`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render About page
-2. Inspect rendered HTML</t>
-  </si>
-  <si>
-    <t>`\n\n` rendered as `&lt;br /&gt;&lt;br /&gt;`; single `\n` between sentences silently collapsed (CP-PI-009, projectInfo.jsx:14). Authors must use double-newlines for paragraph breaks.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_052</t>
-  </si>
-  <si>
-    <t>Long key-point text wraps without horizontal scroll</t>
-  </si>
-  <si>
-    <t>Strapi contains a key-point &gt;300 chars</t>
-  </si>
-  <si>
-    <t>1. Render Key Points page on desktop and mobile viewport</t>
-  </si>
-  <si>
-    <t>Text wraps within container; no horizontal scrollbar appears; layout intact across breakpoints.</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  FUNCTIONAL TESTS  (6)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_018</t>
-  </si>
-  <si>
-    <t>Download a document</t>
-  </si>
-  <si>
-    <t>Documents page lists items</t>
-  </si>
-  <si>
-    <t>1. Click Download on a document</t>
-  </si>
-  <si>
-    <t>Browser initiates download or opens the document in a new tab</t>
-  </si>
-  <si>
-    <t>CP_PROJ_023</t>
-  </si>
-  <si>
-    <t>Click a video plays it inline</t>
-  </si>
-  <si>
-    <t>Video page has at least one item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click a video
-2. Click play</t>
-  </si>
-  <si>
-    <t>Video plays inline using the embedded player; controls work</t>
-  </si>
-  <si>
-    <t>CP_PROJ_024</t>
-  </si>
-  <si>
-    <t>Sharing and Content Source</t>
-  </si>
-  <si>
-    <t>Copy / share section link</t>
-  </si>
-  <si>
-    <t>Any project subpage open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Copy the URL from the address bar
-2. Paste into a new tab while logged in</t>
-  </si>
-  <si>
-    <t>Same section page loads from the copied URL</t>
-  </si>
-  <si>
-    <t>CP_PROJ_042</t>
-  </si>
-  <si>
-    <t>About loads without redirect when CP session active</t>
-  </si>
-  <si>
-    <t>Valid CP JWT in client storage</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/about` directly in a new tab</t>
-  </si>
-  <si>
-    <t>About page renders without redirect to `/login`; Strapi call fires once; no XR backend dependency for content (FSD §6.1).</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  BUSINESS RULE TESTS  (10)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_011</t>
-  </si>
-  <si>
-    <t>About is read-only — no edit controls present</t>
-  </si>
-  <si>
-    <t>1. Inspect page for Edit / Save / Delete actions</t>
-  </si>
-  <si>
-    <t>No edit controls; content is read-only</t>
-  </si>
-  <si>
-    <t>CP_PROJ_016</t>
-  </si>
-  <si>
-    <t>Amenities content is read-only</t>
-  </si>
-  <si>
-    <t>Amenities open</t>
-  </si>
-  <si>
-    <t>1. Look for any input or edit action</t>
-  </si>
-  <si>
-    <t>No editable controls available</t>
-  </si>
-  <si>
-    <t>CP_PROJ_019</t>
-  </si>
-  <si>
-    <t>Documents are read-only — no upload control</t>
-  </si>
-  <si>
-    <t>1. Look for any Upload / Delete control</t>
-  </si>
-  <si>
-    <t>No upload/edit controls visible — content fully read-only</t>
-  </si>
-  <si>
-    <t>CP_PROJ_021</t>
-  </si>
-  <si>
-    <t>Key Points are read-only</t>
-  </si>
-  <si>
-    <t>1. Look for Edit/Add controls</t>
-  </si>
-  <si>
-    <t>No edit controls present</t>
-  </si>
-  <si>
-    <t>CP_PROJ_026</t>
-  </si>
-  <si>
-    <t>All sections accessible regardless of allocation campaign state</t>
-  </si>
-  <si>
-    <t>Allocation campaign is closed for the project</t>
-  </si>
-  <si>
-    <t>1. Open each project section</t>
-  </si>
-  <si>
-    <t>All sections remain accessible to CPs regardless of campaign status</t>
-  </si>
-  <si>
-    <t>CP_PROJ_027</t>
-  </si>
-  <si>
-    <t>Master CP and Member CP have identical access (no per-CP project assignment)</t>
-  </si>
-  <si>
-    <t>Master CP M; Member CP N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Login as M, monitor Strapi requests
-2. Login as N, monitor Strapi requests</t>
-  </si>
-  <si>
-    <t>Both fetch identical content from `&lt;StrapiBase&gt;/api/projects/1?populate=deep`. There is NO CP-project assignment table — every CP sees the same project (CP-PI-003). Document.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_031</t>
-  </si>
-  <si>
-    <t>Project ID hardcoded to `1` regardless of env</t>
-  </si>
-  <si>
-    <t>UAT (backend projectId=2)</t>
-  </si>
-  <si>
-    <t>1. Inspect Strapi URL</t>
-  </si>
-  <si>
-    <t>URL = `&lt;StrapiBase&gt;/api/projects/1?populate=deep` (CP-PI-002, Urls.js:7). Mismatched with backend project resolution — drift if Strapi project 1 differs from backend project 2.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_036</t>
-  </si>
-  <si>
-    <t>No analytics / view tracking on project pages</t>
-  </si>
-  <si>
-    <t>CP browses project pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Browse all sections
-2. Check XR DB / logs for view tracking</t>
-  </si>
-  <si>
-    <t>No tracking exists in XR Portal (QA-Risk-10). If engagement metrics needed, file as gap.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_048</t>
-  </si>
-  <si>
-    <t>Amenities list is identical for Master CP and Member CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Login as M, snapshot amenities list
-2. Login as N, snapshot amenities list
-3. Compare</t>
-  </si>
-  <si>
-    <t>Lists are byte-identical — Strapi has no per-CP scoping; no CP-project assignment table (CP-PI-003). Both fetch same `projects/1?populate=deep`.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_060</t>
-  </si>
-  <si>
-    <t>Videos page is identical for Master CP and Member CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Login as M, list videos
-2. Login as N, list videos</t>
-  </si>
-  <si>
-    <t>Same video list both times — no per-CP scoping in Strapi (CP-PI-003). Confirms no project-assignment table on CP side.</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  INTEGRATION TESTS  (17)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_025</t>
-  </si>
-  <si>
-    <t>Content reflects latest Strapi publish</t>
-  </si>
-  <si>
-    <t>Admin has published an update in Strapi CMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open the affected section in CP portal
-2. Hard refresh</t>
-  </si>
-  <si>
-    <t>Updated content is visible reflecting the latest Strapi publish</t>
-  </si>
-  <si>
-    <t>CP_PROJ_030</t>
-  </si>
-  <si>
-    <t>Frontend fetches Strapi directly (no XR proxy)</t>
-  </si>
-  <si>
-    <t>CP logged in, network tab open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/about`
-2. Inspect network requests</t>
-  </si>
-  <si>
-    <t>Direct `GET &lt;BaseURL&gt;/api/projects/1?populate=deep` to Strapi host. NO request to XR backend `/api/v1/*` for project content (Urls.js:7).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_032</t>
-  </si>
-  <si>
-    <t>Strapi outage breaks CP project pages silently</t>
-  </si>
-  <si>
-    <t>Block Strapi URL in browser</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/about`</t>
-  </si>
-  <si>
-    <t>Frontend fails to render — no XR-side circuit breaker / cache (CP-PI-007). UI may white-screen. Document accessibility implications.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_037</t>
-  </si>
-  <si>
-    <t>About section sources `information` field directly from Strapi</t>
-  </si>
-  <si>
-    <t>CP logged in; About page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to `/project1/about`
-2. Inspect network requests</t>
-  </si>
-  <si>
-    <t>A `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` is fired directly from the CP browser; About content renders from `data.attributes.information` field (CP-PI-002, Urls.js:7). No XR backend call for project content.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_041</t>
-  </si>
-  <si>
-    <t>About reflects latest Strapi publish without hard refresh delay</t>
-  </si>
-  <si>
-    <t>Admin updates `information` in Strapi and clicks Publish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. CP performs hard refresh on `/project1/about` (Ctrl+Shift+R)
-2. Read content</t>
-  </si>
-  <si>
-    <t>Updated content appears immediately — no XR-side ISR/cache (CP-PI-007). Browser fetch hits Strapi live each load.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_043</t>
-  </si>
-  <si>
-    <t>Amenities list sourced from Strapi `amenities` relation</t>
-  </si>
-  <si>
-    <t>Amenities page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/amenities`
-2. Inspect Strapi response</t>
-  </si>
-  <si>
-    <t>Amenity items rendered from `data.attributes.amenities.data[].attributes` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). Each item shows name + icon URL.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_044</t>
-  </si>
-  <si>
-    <t>Amenity icons load from Strapi asset URLs without 404s</t>
-  </si>
-  <si>
-    <t>Strapi amenities have published icon assets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render Amenities list
-2. Observe icon image requests in network tab</t>
-  </si>
-  <si>
-    <t>Every icon URL (raw Strapi `attributes.url`) returns 200; no broken-image placeholders; unsigned URLs cacheable (CP-PI-005).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_046</t>
-  </si>
-  <si>
-    <t>Strapi outage breaks Amenities section silently</t>
-  </si>
-  <si>
-    <t>Block Strapi host in browser DevTools</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/amenities`</t>
-  </si>
-  <si>
-    <t>Frontend has NO XR-side fallback — section either white-screens or shows error boundary (CP-PI-007). No cached version served by XR backend. Document accessibility/UX gap.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_047</t>
-  </si>
-  <si>
-    <t>Amenities returns DRAFT entries via populate=deep (publish gating bug)</t>
-  </si>
-  <si>
-    <t>Admin creates an amenity in Strapi but does NOT publish it</t>
-  </si>
-  <si>
-    <t>1. Open Amenities page in CP</t>
-  </si>
-  <si>
-    <t>Verify whether draft amenity appears. `populate=deep` may include DRAFT + PUBLISHED unless `publicationState=live` is passed (CP-PI-008, QA-Risk-14). If DRAFT visible → document as bug.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_049</t>
-  </si>
-  <si>
-    <t>Key Points sourced from Strapi `keyPoints` field</t>
-  </si>
-  <si>
-    <t>Key Points page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/keyPoints`
-2. Inspect Strapi response</t>
-  </si>
-  <si>
-    <t>List items rendered from `data.attributes.keyPoints` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). No XR backend route involved.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_050</t>
-  </si>
-  <si>
-    <t>Key Points renders ordered list with correct sequence from Strapi</t>
-  </si>
-  <si>
-    <t>Strapi has 5 key-point entries in defined order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render Key Points page
-2. Read items top → bottom</t>
-  </si>
-  <si>
-    <t>Items render in the same order as the Strapi array; no client-side re-sort; numbering / bullets follow source ordering.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_054</t>
-  </si>
-  <si>
-    <t>Key Points reflects latest Strapi publish after hard refresh</t>
-  </si>
-  <si>
-    <t>Admin publishes a new key-point in Strapi</t>
-  </si>
-  <si>
-    <t>1. CP performs Ctrl+Shift+R on `/project1/keyPoints`</t>
-  </si>
-  <si>
-    <t>New point appears immediately — no XR-side cache (CP-PI-007). Browser request hits Strapi live.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_055</t>
-  </si>
-  <si>
-    <t>Videos list sourced from Strapi `videos` relation</t>
-  </si>
-  <si>
-    <t>Videos page open; network tab visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/videos`
-2. Inspect Strapi response</t>
-  </si>
-  <si>
-    <t>Items rendered from `data.attributes.videos.data[]` returned by `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` (Urls.js:7). Each item supplies a video URL/embed code + thumbnail.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_057</t>
-  </si>
-  <si>
-    <t>Video thumbnails load from Strapi asset URLs</t>
-  </si>
-  <si>
-    <t>At least 2 published videos in Strapi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Render Videos page
-2. Inspect each `&lt;img&gt;` request</t>
-  </si>
-  <si>
-    <t>Thumbnail URLs (raw Strapi asset) return 200; no 404s; unsigned URLs cacheable; same external-shareable trait as brochure assets (CP-PI-005).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_058</t>
-  </si>
-  <si>
-    <t>Video embed plays without leaking CP session credentials</t>
-  </si>
-  <si>
-    <t>Video uses third-party embed (YouTube/Vimeo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click and play a video
-2. Inspect outbound requests in network tab</t>
-  </si>
-  <si>
-    <t>Requests go directly to third-party host; no XR JWT / cookies forwarded; embed renders inside iframe sandbox.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_063</t>
-  </si>
-  <si>
-    <t>Strapi DRAFT entries should not leak via `populate=deep`</t>
-  </si>
-  <si>
-    <t>Admin creates a DRAFT entry in any populated relation (gallery/videos/keyPoints/amenities) without publishing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/&lt;section&gt;` as CP
-2. Compare visible items vs Strapi admin</t>
-  </si>
-  <si>
-    <t>Only PUBLISHED entries should render. If DRAFT appears → file as bug (CP-PI-008, QA-Risk-14). Fix is to add `publicationState=live` to Strapi URL.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_064</t>
-  </si>
-  <si>
-    <t>Hard refresh always fetches latest Strapi state (no XR cache)</t>
-  </si>
-  <si>
-    <t>Admin publishes a content edit in Strapi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. CP triggers Ctrl+Shift+R on any project section
-2. Inspect network requests</t>
-  </si>
-  <si>
-    <t>A fresh `GET &lt;StrapiBase&gt;/api/projects/1?populate=deep` is fired (no 304 / cache-hit on XR side); response reflects newly published content (CP-PI-007). Confirms no XR-side ISR / caching.</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  API TESTS  (3)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_028</t>
-  </si>
-  <si>
-    <t>XR backend has NO CP project route (verify by 404)</t>
-  </si>
-  <si>
-    <t>CP JWT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. `GET /api/v1/cp/project` with CP JWT
-2. `GET /api/v1/cp/brochure`
-3. `GET /api/v1/cp/documents`</t>
-  </si>
-  <si>
-    <t>All return 404 — no such routes mounted (FSD §6.1, cp.routes.js verified).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_029</t>
-  </si>
-  <si>
-    <t>CP token rejected on shared commonRoutes</t>
-  </si>
-  <si>
-    <t>Valid CP JWT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. `GET /api/v1/towers` with CP JWT
-2. `GET /api/v1/projects/2/unit-typologies`</t>
-  </si>
-  <si>
-    <t>403 — `cp` role NOT in `restrictTo('user', 'admin', 'sales_manager_admin', 'sales_manager')` (common.routes.js:8).</t>
-  </si>
-  <si>
-    <t>CORRECTION — There is NO XR backend endpoint for CP project info</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  EDGE CASE TESTS  (6)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_014</t>
-  </si>
-  <si>
-    <t>Empty Gallery shows placeholder</t>
-  </si>
-  <si>
-    <t>Strapi returns no images</t>
-  </si>
-  <si>
-    <t>1. Open Gallery</t>
-  </si>
-  <si>
-    <t>Empty-state message such as "No photos available yet" is displayed</t>
-  </si>
-  <si>
-    <t>CP_PROJ_040</t>
-  </si>
-  <si>
-    <t>About section shows empty placeholder when `information` is null</t>
-  </si>
-  <si>
-    <t>Strapi `information` field is null or empty string</t>
-  </si>
-  <si>
-    <t>1. Open About page</t>
-  </si>
-  <si>
-    <t>Page renders heading; body shows empty placeholder or no content paragraph (NOT a JS error or broken layout).</t>
-  </si>
-  <si>
-    <t>CP_PROJ_045</t>
-  </si>
-  <si>
-    <t>Empty Amenities list shows graceful placeholder</t>
-  </si>
-  <si>
-    <t>Strapi returns `amenities.data = []`</t>
-  </si>
-  <si>
-    <t>1. Open Amenities page</t>
-  </si>
-  <si>
-    <t>Friendly empty-state copy displayed (e.g., "No amenities published yet"); UI does not error; section heading still renders.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_051</t>
-  </si>
-  <si>
-    <t>Empty Key Points list shows placeholder</t>
-  </si>
-  <si>
-    <t>Strapi `keyPoints` array is empty</t>
-  </si>
-  <si>
-    <t>1. Open Key Points page</t>
-  </si>
-  <si>
-    <t>Page renders with heading and friendly empty-state copy (e.g., "No key points published yet"); no JS errors.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_056</t>
-  </si>
-  <si>
-    <t>Empty Videos list shows placeholder copy</t>
-  </si>
-  <si>
-    <t>Strapi returns no videos</t>
-  </si>
-  <si>
-    <t>1. Open Videos page</t>
-  </si>
-  <si>
-    <t>Empty-state copy (e.g., "No videos available yet"); section heading still renders; no broken layout.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_059</t>
-  </si>
-  <si>
-    <t>Broken/invalid video URL falls back gracefully</t>
-  </si>
-  <si>
-    <t>A Strapi video item has malformed URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Videos page
-2. Click the broken video</t>
-  </si>
-  <si>
-    <t>Embedded player shows its own error UI (or thumbnail with "Unavailable" overlay); page does not crash; other videos remain playable.</t>
-  </si>
-  <si>
-    <t>━━━━━━━━━━  NEGATIVE TESTS  (7)  ━━━━━━━━━━</t>
-  </si>
-  <si>
-    <t>CP_PROJ_009</t>
-  </si>
-  <si>
-    <t>Logged-out user redirected from project pages</t>
-  </si>
-  <si>
-    <t>1. Open `/project1/about` directly in a fresh browser</t>
-  </si>
-  <si>
-    <t>Redirect to `/login`</t>
-  </si>
-  <si>
-    <t>CP_PROJ_033</t>
-  </si>
-  <si>
-    <t>`information` field XSS via Strapi WYSIWYG (potential)</t>
-  </si>
-  <si>
-    <t>Admin can write to Strapi `information` field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Insert `&lt;script&gt;alert(1)&lt;/script&gt;` via Strapi admin
-2. Open `/project1/projectInfo`</t>
-  </si>
-  <si>
-    <t>Script executes in CP browser — frontend uses `dangerouslySetInnerHTML` without sanitization (CP-PI-004, projectInfo.jsx:14). Trust boundary depends entirely on Strapi authoring controls. Document as security gap.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_034</t>
-  </si>
-  <si>
-    <t>Brochure URL is unsigned Strapi asset (shareable externally)</t>
-  </si>
-  <si>
-    <t>Project info page open with brochure published</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Copy brochure URL from `data.brochure.data.attributes.url`
-2. Open in incognito (no CP session)</t>
-  </si>
-  <si>
-    <t>PDF downloads without auth — raw Strapi URL, no presigned/expiry (CP-PI-005). Confirm with security if acceptable.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_039</t>
-  </si>
-  <si>
-    <t>About content uses dangerouslySetInnerHTML — script tags execute</t>
-  </si>
-  <si>
-    <t>Admin authors `&lt;script&gt;console.log("xss")&lt;/script&gt;` in Strapi `information`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open `/project1/about`
-2. Inspect browser console</t>
-  </si>
-  <si>
-    <t>Script executes — frontend uses `dangerouslySetInnerHTML` without sanitization (CP-PI-004, projectInfo.jsx:14). KNOWN SECURITY GAP: trust boundary lies entirely with Strapi authoring controls.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_053</t>
-  </si>
-  <si>
-    <t>Key Points HTML content uses safe rendering (NOT dangerouslySetInnerHTML)</t>
-  </si>
-  <si>
-    <t>Strapi key-point contains `&lt;script&gt;alert(1)&lt;/script&gt;` string</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open Key Points page
-2. Inspect DOM</t>
-  </si>
-  <si>
-    <t>Script tag rendered as escaped text (NOT executed). If it executes → file as XSS gap analogous to CP_PROJ_033 / CP-PI-004. Verify keyPoints uses safe text rendering.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_061</t>
-  </si>
-  <si>
-    <t>Shared section URL opens to logged-out user redirects to /login</t>
-  </si>
-  <si>
-    <t>CP copies URL of `/project1/amenities` and shares to logged-out user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open shared URL in incognito window
-2. Observe behaviour</t>
-  </si>
-  <si>
-    <t>App shell route guard redirects to `/login` before fetching Strapi content (frontend-only redirect; no XR session check). After login, user routes back to original path.</t>
-  </si>
-  <si>
-    <t>CP_PROJ_062</t>
-  </si>
-  <si>
-    <t>Brochure URL copied externally still serves PDF (no auth)</t>
-  </si>
-  <si>
-    <t>CP copies brochure URL from `data.brochure.data.attributes.url`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open URL in incognito browser (no CP session)
-2. Observe</t>
-  </si>
-  <si>
-    <t>PDF downloads/renders directly from Strapi without auth — raw asset URL with no expiry / signature (CP-PI-005). Document risk; confirm with security if acceptable.</t>
   </si>
 </sst>
 </file>
@@ -28373,3394 +27372,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:O76"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="46" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="38" customWidth="1"/>
-    <col min="14" max="14" width="32" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>2170</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>1734</v>
-      </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-    </row>
-    <row r="4" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>2171</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>2173</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>862</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>2174</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>2175</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J4" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L4" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M4" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O4" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
-        <v>2176</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>2177</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>2178</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>2179</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>2180</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L5" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N5" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O5" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>2181</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>2182</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>526</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>2183</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>2184</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L6" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="M6" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="N6" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="O6" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
-        <v>2185</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>2186</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>526</v>
-      </c>
-      <c r="F7" s="17" t="s">
-        <v>2187</v>
-      </c>
-      <c r="G7" s="17" t="s">
-        <v>2188</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J7" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K7" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M7" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O7" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
-        <v>2189</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>2190</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>526</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>2191</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>2192</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K8" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M8" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N8" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O8" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>2193</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>2194</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>526</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>2195</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>2196</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="K9" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L9" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="O9" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
-        <v>2197</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>2198</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>526</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>2199</v>
-      </c>
-      <c r="G10" s="20" t="s">
-        <v>2200</v>
-      </c>
-      <c r="H10" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J10" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K10" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L10" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M10" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N10" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O10" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
-        <v>2201</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>2202</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>526</v>
-      </c>
-      <c r="F11" s="17" t="s">
-        <v>2203</v>
-      </c>
-      <c r="G11" s="17" t="s">
-        <v>2204</v>
-      </c>
-      <c r="H11" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J11" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K11" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L11" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M11" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N11" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O11" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>2205</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>2207</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>2208</v>
-      </c>
-      <c r="F12" s="17" t="s">
-        <v>2209</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>2210</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I12" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J12" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K12" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L12" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M12" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N12" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O12" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
-        <v>2211</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>2212</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>2213</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>2214</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>2215</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>2216</v>
-      </c>
-      <c r="H13" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I13" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J13" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K13" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L13" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M13" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N13" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O13" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>2217</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>2212</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>2218</v>
-      </c>
-      <c r="E14" s="20" t="s">
-        <v>2219</v>
-      </c>
-      <c r="F14" s="20" t="s">
-        <v>2220</v>
-      </c>
-      <c r="G14" s="20" t="s">
-        <v>2221</v>
-      </c>
-      <c r="H14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J14" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K14" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L14" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O14" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
-        <v>2222</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>2224</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>2225</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>2226</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>2227</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J15" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K15" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L15" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M15" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N15" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O15" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>2228</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>2229</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>2230</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>2231</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>2232</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>2233</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I16" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="J16" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="K16" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L16" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="M16" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="N16" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="O16" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>2234</v>
-      </c>
-      <c r="B17" s="17" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>2236</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>2237</v>
-      </c>
-      <c r="F17" s="17" t="s">
-        <v>2238</v>
-      </c>
-      <c r="G17" s="17" t="s">
-        <v>2239</v>
-      </c>
-      <c r="H17" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I17" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J17" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K17" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L17" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M17" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N17" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O17" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
-        <v>2240</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>2242</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>2243</v>
-      </c>
-      <c r="F18" s="17" t="s">
-        <v>2244</v>
-      </c>
-      <c r="G18" s="17" t="s">
-        <v>2245</v>
-      </c>
-      <c r="H18" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I18" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J18" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K18" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L18" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M18" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N18" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O18" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>2246</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>2247</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>2248</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>2249</v>
-      </c>
-      <c r="G19" s="20" t="s">
-        <v>2250</v>
-      </c>
-      <c r="H19" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I19" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J19" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K19" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L19" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M19" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N19" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O19" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
-        <v>2251</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>2252</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>2253</v>
-      </c>
-      <c r="F20" s="20" t="s">
-        <v>2254</v>
-      </c>
-      <c r="G20" s="20" t="s">
-        <v>2255</v>
-      </c>
-      <c r="H20" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I20" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J20" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K20" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L20" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M20" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N20" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O20" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
-        <v>2256</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>2257</v>
-      </c>
-      <c r="E21" s="20" t="s">
-        <v>2258</v>
-      </c>
-      <c r="F21" s="20" t="s">
-        <v>2259</v>
-      </c>
-      <c r="G21" s="20" t="s">
-        <v>2260</v>
-      </c>
-      <c r="H21" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I21" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J21" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K21" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L21" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M21" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N21" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O21" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
-        <v>2261</v>
-      </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-    </row>
-    <row r="23" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="G23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="H23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="K23" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L23" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N23" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O23" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
-        <v>2262</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>2229</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>2263</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>2264</v>
-      </c>
-      <c r="F24" s="17" t="s">
-        <v>2265</v>
-      </c>
-      <c r="G24" s="17" t="s">
-        <v>2266</v>
-      </c>
-      <c r="H24" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I24" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J24" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K24" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L24" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M24" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N24" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O24" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="25" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
-        <v>2267</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>2268</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>2269</v>
-      </c>
-      <c r="F25" s="20" t="s">
-        <v>2270</v>
-      </c>
-      <c r="G25" s="20" t="s">
-        <v>2271</v>
-      </c>
-      <c r="H25" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I25" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J25" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K25" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L25" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M25" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N25" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O25" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="19" t="s">
-        <v>2272</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="D26" s="20" t="s">
-        <v>2274</v>
-      </c>
-      <c r="E26" s="20" t="s">
-        <v>2275</v>
-      </c>
-      <c r="F26" s="20" t="s">
-        <v>2276</v>
-      </c>
-      <c r="G26" s="20" t="s">
-        <v>2277</v>
-      </c>
-      <c r="H26" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I26" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J26" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K26" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L26" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M26" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N26" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O26" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
-        <v>2278</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>2279</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>2280</v>
-      </c>
-      <c r="F27" s="17" t="s">
-        <v>2281</v>
-      </c>
-      <c r="G27" s="17" t="s">
-        <v>2282</v>
-      </c>
-      <c r="H27" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I27" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J27" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K27" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L27" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M27" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N27" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O27" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>148</v>
-      </c>
-      <c r="E28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="F28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="G28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="H28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="K28" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L28" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N28" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O28" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>2283</v>
-      </c>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
-      <c r="O29" s="11"/>
-    </row>
-    <row r="30" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
-        <v>2284</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>2285</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>2208</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>2286</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>2287</v>
-      </c>
-      <c r="H30" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="K30" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L30" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="M30" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="N30" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="O30" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="31" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
-        <v>2288</v>
-      </c>
-      <c r="B31" s="20" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>2289</v>
-      </c>
-      <c r="E31" s="20" t="s">
-        <v>2290</v>
-      </c>
-      <c r="F31" s="20" t="s">
-        <v>2291</v>
-      </c>
-      <c r="G31" s="20" t="s">
-        <v>2292</v>
-      </c>
-      <c r="H31" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J31" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K31" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L31" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M31" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N31" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O31" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="32" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
-        <v>2293</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>2229</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>2294</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>2231</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>2295</v>
-      </c>
-      <c r="G32" s="13" t="s">
-        <v>2296</v>
-      </c>
-      <c r="H32" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I32" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="J32" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="K32" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L32" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="M32" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="N32" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="O32" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="33" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="19" t="s">
-        <v>2297</v>
-      </c>
-      <c r="B33" s="20" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>2298</v>
-      </c>
-      <c r="E33" s="20" t="s">
-        <v>2237</v>
-      </c>
-      <c r="F33" s="20" t="s">
-        <v>2299</v>
-      </c>
-      <c r="G33" s="20" t="s">
-        <v>2300</v>
-      </c>
-      <c r="H33" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J33" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K33" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L33" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M33" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N33" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O33" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
-        <v>2301</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C34" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>2302</v>
-      </c>
-      <c r="E34" s="20" t="s">
-        <v>2303</v>
-      </c>
-      <c r="F34" s="20" t="s">
-        <v>2304</v>
-      </c>
-      <c r="G34" s="20" t="s">
-        <v>2305</v>
-      </c>
-      <c r="H34" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I34" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J34" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K34" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L34" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M34" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N34" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O34" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="35" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
-        <v>2306</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>2307</v>
-      </c>
-      <c r="E35" s="20" t="s">
-        <v>2308</v>
-      </c>
-      <c r="F35" s="20" t="s">
-        <v>2309</v>
-      </c>
-      <c r="G35" s="20" t="s">
-        <v>2310</v>
-      </c>
-      <c r="H35" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I35" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J35" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K35" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L35" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M35" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N35" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O35" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
-        <v>2311</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C36" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D36" s="20" t="s">
-        <v>2312</v>
-      </c>
-      <c r="E36" s="20" t="s">
-        <v>2313</v>
-      </c>
-      <c r="F36" s="20" t="s">
-        <v>2314</v>
-      </c>
-      <c r="G36" s="20" t="s">
-        <v>2315</v>
-      </c>
-      <c r="H36" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I36" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J36" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K36" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L36" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M36" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N36" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O36" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
-        <v>2316</v>
-      </c>
-      <c r="B37" s="20" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>2317</v>
-      </c>
-      <c r="E37" s="20" t="s">
-        <v>2318</v>
-      </c>
-      <c r="F37" s="20" t="s">
-        <v>2319</v>
-      </c>
-      <c r="G37" s="20" t="s">
-        <v>2320</v>
-      </c>
-      <c r="H37" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I37" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J37" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K37" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L37" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M37" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N37" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O37" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="38" ht="60" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
-        <v>2321</v>
-      </c>
-      <c r="B38" s="20" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>2322</v>
-      </c>
-      <c r="E38" s="20" t="s">
-        <v>2308</v>
-      </c>
-      <c r="F38" s="20" t="s">
-        <v>2323</v>
-      </c>
-      <c r="G38" s="20" t="s">
-        <v>2324</v>
-      </c>
-      <c r="H38" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I38" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J38" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K38" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L38" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M38" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N38" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O38" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="19" t="s">
-        <v>2325</v>
-      </c>
-      <c r="B39" s="20" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C39" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="D39" s="20" t="s">
-        <v>2326</v>
-      </c>
-      <c r="E39" s="20" t="s">
-        <v>2308</v>
-      </c>
-      <c r="F39" s="20" t="s">
-        <v>2327</v>
-      </c>
-      <c r="G39" s="20" t="s">
-        <v>2328</v>
-      </c>
-      <c r="H39" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I39" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J39" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K39" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L39" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M39" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N39" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O39" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="11" t="s">
-        <v>2329</v>
-      </c>
-      <c r="B40" s="11"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="11"/>
-      <c r="J40" s="11"/>
-      <c r="K40" s="11"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="11"/>
-      <c r="N40" s="11"/>
-      <c r="O40" s="11"/>
-    </row>
-    <row r="41" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
-        <v>2330</v>
-      </c>
-      <c r="B41" s="17" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C41" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D41" s="17" t="s">
-        <v>2331</v>
-      </c>
-      <c r="E41" s="17" t="s">
-        <v>2332</v>
-      </c>
-      <c r="F41" s="17" t="s">
-        <v>2333</v>
-      </c>
-      <c r="G41" s="17" t="s">
-        <v>2334</v>
-      </c>
-      <c r="H41" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I41" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J41" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K41" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L41" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M41" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N41" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O41" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="42" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
-        <v>2335</v>
-      </c>
-      <c r="B42" s="17" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C42" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D42" s="17" t="s">
-        <v>2336</v>
-      </c>
-      <c r="E42" s="17" t="s">
-        <v>2337</v>
-      </c>
-      <c r="F42" s="17" t="s">
-        <v>2338</v>
-      </c>
-      <c r="G42" s="17" t="s">
-        <v>2339</v>
-      </c>
-      <c r="H42" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I42" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J42" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K42" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L42" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M42" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N42" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O42" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="19" t="s">
-        <v>2340</v>
-      </c>
-      <c r="B43" s="20" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C43" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D43" s="20" t="s">
-        <v>2341</v>
-      </c>
-      <c r="E43" s="20" t="s">
-        <v>2342</v>
-      </c>
-      <c r="F43" s="20" t="s">
-        <v>2343</v>
-      </c>
-      <c r="G43" s="20" t="s">
-        <v>2344</v>
-      </c>
-      <c r="H43" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I43" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J43" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K43" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L43" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M43" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N43" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O43" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
-        <v>2345</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C44" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D44" s="17" t="s">
-        <v>2346</v>
-      </c>
-      <c r="E44" s="17" t="s">
-        <v>2347</v>
-      </c>
-      <c r="F44" s="17" t="s">
-        <v>2348</v>
-      </c>
-      <c r="G44" s="17" t="s">
-        <v>2349</v>
-      </c>
-      <c r="H44" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I44" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J44" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K44" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L44" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M44" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N44" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O44" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
-        <v>2350</v>
-      </c>
-      <c r="B45" s="17" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C45" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D45" s="17" t="s">
-        <v>2351</v>
-      </c>
-      <c r="E45" s="17" t="s">
-        <v>2352</v>
-      </c>
-      <c r="F45" s="17" t="s">
-        <v>2353</v>
-      </c>
-      <c r="G45" s="17" t="s">
-        <v>2354</v>
-      </c>
-      <c r="H45" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I45" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J45" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K45" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L45" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M45" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N45" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O45" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
-        <v>2355</v>
-      </c>
-      <c r="B46" s="17" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C46" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D46" s="17" t="s">
-        <v>2356</v>
-      </c>
-      <c r="E46" s="17" t="s">
-        <v>2357</v>
-      </c>
-      <c r="F46" s="17" t="s">
-        <v>2358</v>
-      </c>
-      <c r="G46" s="17" t="s">
-        <v>2359</v>
-      </c>
-      <c r="H46" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I46" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J46" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K46" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L46" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M46" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N46" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O46" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="47" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47" s="19" t="s">
-        <v>2360</v>
-      </c>
-      <c r="B47" s="20" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C47" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D47" s="20" t="s">
-        <v>2361</v>
-      </c>
-      <c r="E47" s="20" t="s">
-        <v>2362</v>
-      </c>
-      <c r="F47" s="20" t="s">
-        <v>2363</v>
-      </c>
-      <c r="G47" s="20" t="s">
-        <v>2364</v>
-      </c>
-      <c r="H47" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I47" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J47" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K47" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L47" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M47" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N47" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O47" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="48" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
-        <v>2365</v>
-      </c>
-      <c r="B48" s="20" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C48" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D48" s="20" t="s">
-        <v>2366</v>
-      </c>
-      <c r="E48" s="20" t="s">
-        <v>2367</v>
-      </c>
-      <c r="F48" s="20" t="s">
-        <v>2368</v>
-      </c>
-      <c r="G48" s="20" t="s">
-        <v>2369</v>
-      </c>
-      <c r="H48" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I48" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J48" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K48" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L48" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M48" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N48" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O48" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
-        <v>2370</v>
-      </c>
-      <c r="B49" s="17" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C49" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D49" s="17" t="s">
-        <v>2371</v>
-      </c>
-      <c r="E49" s="17" t="s">
-        <v>2372</v>
-      </c>
-      <c r="F49" s="17" t="s">
-        <v>2373</v>
-      </c>
-      <c r="G49" s="17" t="s">
-        <v>2374</v>
-      </c>
-      <c r="H49" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I49" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J49" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K49" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L49" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M49" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N49" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O49" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50" s="16" t="s">
-        <v>2375</v>
-      </c>
-      <c r="B50" s="17" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C50" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D50" s="17" t="s">
-        <v>2376</v>
-      </c>
-      <c r="E50" s="17" t="s">
-        <v>2377</v>
-      </c>
-      <c r="F50" s="17" t="s">
-        <v>2378</v>
-      </c>
-      <c r="G50" s="17" t="s">
-        <v>2379</v>
-      </c>
-      <c r="H50" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I50" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J50" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K50" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L50" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M50" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N50" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O50" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51" s="19" t="s">
-        <v>2380</v>
-      </c>
-      <c r="B51" s="20" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C51" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D51" s="20" t="s">
-        <v>2381</v>
-      </c>
-      <c r="E51" s="20" t="s">
-        <v>2382</v>
-      </c>
-      <c r="F51" s="20" t="s">
-        <v>2383</v>
-      </c>
-      <c r="G51" s="20" t="s">
-        <v>2384</v>
-      </c>
-      <c r="H51" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I51" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J51" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K51" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L51" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M51" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N51" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O51" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="52" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52" s="16" t="s">
-        <v>2385</v>
-      </c>
-      <c r="B52" s="17" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D52" s="17" t="s">
-        <v>2386</v>
-      </c>
-      <c r="E52" s="17" t="s">
-        <v>2387</v>
-      </c>
-      <c r="F52" s="17" t="s">
-        <v>2388</v>
-      </c>
-      <c r="G52" s="17" t="s">
-        <v>2389</v>
-      </c>
-      <c r="H52" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I52" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J52" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K52" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L52" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M52" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N52" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O52" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53" s="16" t="s">
-        <v>2390</v>
-      </c>
-      <c r="B53" s="17" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D53" s="17" t="s">
-        <v>2391</v>
-      </c>
-      <c r="E53" s="17" t="s">
-        <v>2392</v>
-      </c>
-      <c r="F53" s="17" t="s">
-        <v>2393</v>
-      </c>
-      <c r="G53" s="17" t="s">
-        <v>2394</v>
-      </c>
-      <c r="H53" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I53" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J53" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K53" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L53" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M53" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N53" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O53" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="19" t="s">
-        <v>2395</v>
-      </c>
-      <c r="B54" s="20" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C54" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D54" s="20" t="s">
-        <v>2396</v>
-      </c>
-      <c r="E54" s="20" t="s">
-        <v>2397</v>
-      </c>
-      <c r="F54" s="20" t="s">
-        <v>2398</v>
-      </c>
-      <c r="G54" s="20" t="s">
-        <v>2399</v>
-      </c>
-      <c r="H54" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I54" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J54" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K54" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L54" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M54" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N54" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O54" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="19" t="s">
-        <v>2400</v>
-      </c>
-      <c r="B55" s="20" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C55" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D55" s="20" t="s">
-        <v>2401</v>
-      </c>
-      <c r="E55" s="20" t="s">
-        <v>2402</v>
-      </c>
-      <c r="F55" s="20" t="s">
-        <v>2403</v>
-      </c>
-      <c r="G55" s="20" t="s">
-        <v>2404</v>
-      </c>
-      <c r="H55" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I55" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J55" s="20" t="s">
-        <v>1873</v>
-      </c>
-      <c r="K55" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L55" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M55" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N55" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O55" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="16" t="s">
-        <v>2405</v>
-      </c>
-      <c r="B56" s="17" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C56" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D56" s="17" t="s">
-        <v>2406</v>
-      </c>
-      <c r="E56" s="17" t="s">
-        <v>2407</v>
-      </c>
-      <c r="F56" s="17" t="s">
-        <v>2408</v>
-      </c>
-      <c r="G56" s="17" t="s">
-        <v>2409</v>
-      </c>
-      <c r="H56" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I56" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J56" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K56" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L56" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M56" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N56" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O56" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="19" t="s">
-        <v>2410</v>
-      </c>
-      <c r="B57" s="20" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C57" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="D57" s="20" t="s">
-        <v>2411</v>
-      </c>
-      <c r="E57" s="20" t="s">
-        <v>2412</v>
-      </c>
-      <c r="F57" s="20" t="s">
-        <v>2413</v>
-      </c>
-      <c r="G57" s="20" t="s">
-        <v>2414</v>
-      </c>
-      <c r="H57" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I57" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J57" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K57" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L57" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M57" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N57" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O57" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="11" t="s">
-        <v>2415</v>
-      </c>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="11"/>
-      <c r="G58" s="11"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="11"/>
-      <c r="J58" s="11"/>
-      <c r="K58" s="11"/>
-      <c r="L58" s="11"/>
-      <c r="M58" s="11"/>
-      <c r="N58" s="11"/>
-      <c r="O58" s="11"/>
-    </row>
-    <row r="59" ht="60" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="16" t="s">
-        <v>2416</v>
-      </c>
-      <c r="B59" s="17" t="s">
-        <v>2229</v>
-      </c>
-      <c r="C59" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="D59" s="17" t="s">
-        <v>2417</v>
-      </c>
-      <c r="E59" s="17" t="s">
-        <v>2418</v>
-      </c>
-      <c r="F59" s="17" t="s">
-        <v>2419</v>
-      </c>
-      <c r="G59" s="17" t="s">
-        <v>2420</v>
-      </c>
-      <c r="H59" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I59" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J59" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K59" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L59" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M59" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N59" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O59" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="19" t="s">
-        <v>2421</v>
-      </c>
-      <c r="B60" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C60" s="21" t="s">
-        <v>230</v>
-      </c>
-      <c r="D60" s="20" t="s">
-        <v>2422</v>
-      </c>
-      <c r="E60" s="20" t="s">
-        <v>2423</v>
-      </c>
-      <c r="F60" s="20" t="s">
-        <v>2424</v>
-      </c>
-      <c r="G60" s="20" t="s">
-        <v>2425</v>
-      </c>
-      <c r="H60" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I60" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J60" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="K60" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L60" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M60" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N60" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O60" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="61" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A61" s="19" t="s">
-        <v>1442</v>
-      </c>
-      <c r="B61" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C61" s="21" t="s">
-        <v>230</v>
-      </c>
-      <c r="D61" s="20" t="s">
-        <v>2426</v>
-      </c>
-      <c r="E61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="F61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="G61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="H61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="K61" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L61" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N61" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O61" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="62" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A62" s="11" t="s">
-        <v>2427</v>
-      </c>
-      <c r="B62" s="11"/>
-      <c r="C62" s="11"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="11"/>
-      <c r="F62" s="11"/>
-      <c r="G62" s="11"/>
-      <c r="H62" s="11"/>
-      <c r="I62" s="11"/>
-      <c r="J62" s="11"/>
-      <c r="K62" s="11"/>
-      <c r="L62" s="11"/>
-      <c r="M62" s="11"/>
-      <c r="N62" s="11"/>
-      <c r="O62" s="11"/>
-    </row>
-    <row r="63" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A63" s="19" t="s">
-        <v>2428</v>
-      </c>
-      <c r="B63" s="20" t="s">
-        <v>2212</v>
-      </c>
-      <c r="C63" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D63" s="20" t="s">
-        <v>2429</v>
-      </c>
-      <c r="E63" s="20" t="s">
-        <v>2430</v>
-      </c>
-      <c r="F63" s="20" t="s">
-        <v>2431</v>
-      </c>
-      <c r="G63" s="20" t="s">
-        <v>2432</v>
-      </c>
-      <c r="H63" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I63" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J63" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K63" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L63" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M63" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N63" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O63" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="64" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A64" s="19" t="s">
-        <v>2433</v>
-      </c>
-      <c r="B64" s="20" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C64" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D64" s="20" t="s">
-        <v>2434</v>
-      </c>
-      <c r="E64" s="20" t="s">
-        <v>2435</v>
-      </c>
-      <c r="F64" s="20" t="s">
-        <v>2436</v>
-      </c>
-      <c r="G64" s="20" t="s">
-        <v>2437</v>
-      </c>
-      <c r="H64" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I64" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J64" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K64" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L64" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M64" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N64" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O64" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A65" s="19" t="s">
-        <v>2438</v>
-      </c>
-      <c r="B65" s="20" t="s">
-        <v>2223</v>
-      </c>
-      <c r="C65" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D65" s="20" t="s">
-        <v>2439</v>
-      </c>
-      <c r="E65" s="20" t="s">
-        <v>2440</v>
-      </c>
-      <c r="F65" s="20" t="s">
-        <v>2441</v>
-      </c>
-      <c r="G65" s="20" t="s">
-        <v>2442</v>
-      </c>
-      <c r="H65" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I65" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J65" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K65" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L65" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M65" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N65" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O65" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="66" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A66" s="19" t="s">
-        <v>2443</v>
-      </c>
-      <c r="B66" s="20" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C66" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D66" s="20" t="s">
-        <v>2444</v>
-      </c>
-      <c r="E66" s="20" t="s">
-        <v>2445</v>
-      </c>
-      <c r="F66" s="20" t="s">
-        <v>2446</v>
-      </c>
-      <c r="G66" s="20" t="s">
-        <v>2447</v>
-      </c>
-      <c r="H66" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I66" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J66" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K66" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L66" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M66" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N66" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O66" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="67" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" s="19" t="s">
-        <v>2448</v>
-      </c>
-      <c r="B67" s="20" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C67" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D67" s="20" t="s">
-        <v>2449</v>
-      </c>
-      <c r="E67" s="20" t="s">
-        <v>2450</v>
-      </c>
-      <c r="F67" s="20" t="s">
-        <v>2451</v>
-      </c>
-      <c r="G67" s="20" t="s">
-        <v>2452</v>
-      </c>
-      <c r="H67" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I67" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J67" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="K67" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L67" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M67" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N67" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O67" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="68" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A68" s="19" t="s">
-        <v>2453</v>
-      </c>
-      <c r="B68" s="20" t="s">
-        <v>2241</v>
-      </c>
-      <c r="C68" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D68" s="20" t="s">
-        <v>2454</v>
-      </c>
-      <c r="E68" s="20" t="s">
-        <v>2455</v>
-      </c>
-      <c r="F68" s="20" t="s">
-        <v>2456</v>
-      </c>
-      <c r="G68" s="20" t="s">
-        <v>2457</v>
-      </c>
-      <c r="H68" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I68" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J68" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="K68" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L68" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M68" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N68" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O68" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="69" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A69" s="11" t="s">
-        <v>2458</v>
-      </c>
-      <c r="B69" s="11"/>
-      <c r="C69" s="11"/>
-      <c r="D69" s="11"/>
-      <c r="E69" s="11"/>
-      <c r="F69" s="11"/>
-      <c r="G69" s="11"/>
-      <c r="H69" s="11"/>
-      <c r="I69" s="11"/>
-      <c r="J69" s="11"/>
-      <c r="K69" s="11"/>
-      <c r="L69" s="11"/>
-      <c r="M69" s="11"/>
-      <c r="N69" s="11"/>
-      <c r="O69" s="11"/>
-    </row>
-    <row r="70" ht="40" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A70" s="16" t="s">
-        <v>2459</v>
-      </c>
-      <c r="B70" s="17" t="s">
-        <v>2172</v>
-      </c>
-      <c r="C70" s="18" t="s">
-        <v>277</v>
-      </c>
-      <c r="D70" s="17" t="s">
-        <v>2460</v>
-      </c>
-      <c r="E70" s="17" t="s">
-        <v>1493</v>
-      </c>
-      <c r="F70" s="17" t="s">
-        <v>2461</v>
-      </c>
-      <c r="G70" s="17" t="s">
-        <v>2462</v>
-      </c>
-      <c r="H70" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I70" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J70" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K70" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L70" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M70" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N70" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O70" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="71" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A71" s="19" t="s">
-        <v>2463</v>
-      </c>
-      <c r="B71" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C71" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D71" s="20" t="s">
-        <v>2464</v>
-      </c>
-      <c r="E71" s="20" t="s">
-        <v>2465</v>
-      </c>
-      <c r="F71" s="20" t="s">
-        <v>2466</v>
-      </c>
-      <c r="G71" s="20" t="s">
-        <v>2467</v>
-      </c>
-      <c r="H71" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I71" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J71" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="K71" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L71" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M71" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N71" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O71" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="72" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A72" s="19" t="s">
-        <v>2468</v>
-      </c>
-      <c r="B72" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C72" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D72" s="20" t="s">
-        <v>2469</v>
-      </c>
-      <c r="E72" s="20" t="s">
-        <v>2470</v>
-      </c>
-      <c r="F72" s="20" t="s">
-        <v>2471</v>
-      </c>
-      <c r="G72" s="20" t="s">
-        <v>2472</v>
-      </c>
-      <c r="H72" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I72" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J72" s="20" t="s">
-        <v>1873</v>
-      </c>
-      <c r="K72" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L72" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M72" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N72" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O72" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="73" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A73" s="19" t="s">
-        <v>2473</v>
-      </c>
-      <c r="B73" s="20" t="s">
-        <v>2206</v>
-      </c>
-      <c r="C73" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D73" s="20" t="s">
-        <v>2474</v>
-      </c>
-      <c r="E73" s="20" t="s">
-        <v>2475</v>
-      </c>
-      <c r="F73" s="20" t="s">
-        <v>2476</v>
-      </c>
-      <c r="G73" s="20" t="s">
-        <v>2477</v>
-      </c>
-      <c r="H73" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I73" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J73" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="K73" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="L73" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M73" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N73" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O73" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="74" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A74" s="19" t="s">
-        <v>2478</v>
-      </c>
-      <c r="B74" s="20" t="s">
-        <v>2235</v>
-      </c>
-      <c r="C74" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D74" s="20" t="s">
-        <v>2479</v>
-      </c>
-      <c r="E74" s="20" t="s">
-        <v>2480</v>
-      </c>
-      <c r="F74" s="20" t="s">
-        <v>2481</v>
-      </c>
-      <c r="G74" s="20" t="s">
-        <v>2482</v>
-      </c>
-      <c r="H74" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I74" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J74" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="K74" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L74" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M74" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N74" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O74" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="75" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A75" s="16" t="s">
-        <v>2483</v>
-      </c>
-      <c r="B75" s="17" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C75" s="18" t="s">
-        <v>277</v>
-      </c>
-      <c r="D75" s="17" t="s">
-        <v>2484</v>
-      </c>
-      <c r="E75" s="17" t="s">
-        <v>2485</v>
-      </c>
-      <c r="F75" s="17" t="s">
-        <v>2486</v>
-      </c>
-      <c r="G75" s="17" t="s">
-        <v>2487</v>
-      </c>
-      <c r="H75" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I75" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="J75" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="K75" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L75" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="M75" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="N75" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="O75" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="76" ht="44" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A76" s="19" t="s">
-        <v>2488</v>
-      </c>
-      <c r="B76" s="20" t="s">
-        <v>2273</v>
-      </c>
-      <c r="C76" s="21" t="s">
-        <v>277</v>
-      </c>
-      <c r="D76" s="20" t="s">
-        <v>2489</v>
-      </c>
-      <c r="E76" s="20" t="s">
-        <v>2490</v>
-      </c>
-      <c r="F76" s="20" t="s">
-        <v>2491</v>
-      </c>
-      <c r="G76" s="20" t="s">
-        <v>2492</v>
-      </c>
-      <c r="H76" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I76" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J76" s="20" t="s">
-        <v>1873</v>
-      </c>
-      <c r="K76" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L76" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="M76" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="N76" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="O76" s="20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A2:O2"/>
-  <mergeCells count="8">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A3:O3"/>
-    <mergeCell ref="A22:O22"/>
-    <mergeCell ref="A29:O29"/>
-    <mergeCell ref="A40:O40"/>
-    <mergeCell ref="A58:O58"/>
-    <mergeCell ref="A62:O62"/>
-    <mergeCell ref="A69:O69"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-</worksheet>
 </file>
</xml_diff>